<commit_message>
fix: improve rescue workbook import layout
</commit_message>
<xml_diff>
--- a/public/downloads/ryutter-deadline-rescue.xlsx
+++ b/public/downloads/ryutter-deadline-rescue.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R617f66595f9f4610"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の3件" sheetId="2" r:id="R6a949612e9cd4c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="課題入力" sheetId="3" r:id="R9f2247bc8f5c44f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RYUTTER取込" sheetId="4" r:id="R233f6bec9815451d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="Rad9360aef01f4a21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の3件" sheetId="2" r:id="R3c26562779d144fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="課題入力" sheetId="3" r:id="R26e60e2a2fd74c31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RYUTTER取込" sheetId="4" r:id="R194eb13ea60b41d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -70,7 +70,7 @@
     <x:numFmt numFmtId="203" formatCode="yyyy/m/d"/>
     <x:numFmt numFmtId="204" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="21">
+  <x:fonts count="24">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Arial"/>
@@ -188,8 +188,25 @@
       <x:color rgb="FF0432FF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF20243A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FF44318D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF373354"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -261,8 +278,23 @@
         <x:fgColor rgb="FFF3F0FF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F0FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF44318D"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="14">
+  <x:borders count="20">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -386,11 +418,53 @@
         <x:color rgb="FFD9E0E6"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD7CEF7"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="115">
+  <x:cellXfs count="144">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -729,6 +803,93 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="16" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="15" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="15" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -12673,9 +12834,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -12683,2248 +12844,2250 @@
       <x:c r="B1" s="49"/>
       <x:c r="C1" s="49"/>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="50" t="str">
-        <x:v>RYUTTER取込</x:v>
-      </x:c>
-      <x:c r="B2" s="49"/>
-      <x:c r="C2" s="49"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="59" t="str">
-        <x:v>下の2列をコピーして、RYUTTERの取り込み画面へ貼り付けます。完了済み・入力不足は表示しません。</x:v>
-      </x:c>
-      <x:c r="B3" s="59" t="str"/>
-      <x:c r="C3" s="59" t="str"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="49"/>
-      <x:c r="B4" s="49"/>
-      <x:c r="C4" s="49"/>
+    <x:row r="2" ht="38" customHeight="1">
+      <x:c r="A2" s="121" t="str">
+        <x:v>RYUTTERへ取り込む</x:v>
+      </x:c>
+      <x:c r="B2" s="121"/>
+      <x:c r="C2" s="121"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="126" t="str">
+        <x:v>① 課題名・締切日をコピー
+② RYUTTERの「課題をまとめて取り込む」へ貼り付け</x:v>
+      </x:c>
+      <x:c r="B3" s="127" t="str"/>
+      <x:c r="C3" s="128" t="str"/>
+    </x:row>
+    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="A4" s="132"/>
+      <x:c r="B4" s="133"/>
+      <x:c r="C4" s="134"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="110" t="str">
+      <x:c r="A5" s="137" t="str">
         <x:v>課題名</x:v>
       </x:c>
-      <x:c r="B5" s="110" t="str">
+      <x:c r="B5" s="137" t="str">
         <x:v>締切日</x:v>
       </x:c>
-      <x:c r="C5" s="110" t="str">
+      <x:c r="C5" s="137" t="str">
         <x:v>状態</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="112" t="str">
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="141" t="str">
         <x:f>IF('課題入力'!H6=1,'課題入力'!A6,"")</x:f>
         <x:v>見本：英語レポート</x:v>
       </x:c>
-      <x:c r="B6" s="113" t="n">
+      <x:c r="B6" s="142" t="n">
         <x:f>IF(A6="","",'課題入力'!B6)</x:f>
         <x:v>46272</x:v>
       </x:c>
-      <x:c r="C6" s="114" t="str">
+      <x:c r="C6" s="143" t="str">
         <x:f>IF(A6="","",'課題入力'!E6)</x:f>
         <x:v>3日以内</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="112" t="str">
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="141" t="str">
         <x:f>IF('課題入力'!H7=1,'課題入力'!A7,"")</x:f>
         <x:v>見本：統計の演習</x:v>
       </x:c>
-      <x:c r="B7" s="113" t="n">
+      <x:c r="B7" s="142" t="n">
         <x:f>IF(A7="","",'課題入力'!B7)</x:f>
         <x:v>46274</x:v>
       </x:c>
-      <x:c r="C7" s="114" t="str">
+      <x:c r="C7" s="143" t="str">
         <x:f>IF(A7="","",'課題入力'!E7)</x:f>
         <x:v>3日以内</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="112" t="str">
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="141" t="str">
         <x:f>IF('課題入力'!H8=1,'課題入力'!A8,"")</x:f>
         <x:v>見本：ゼミの資料</x:v>
       </x:c>
-      <x:c r="B8" s="113" t="n">
+      <x:c r="B8" s="142" t="n">
         <x:f>IF(A8="","",'課題入力'!B8)</x:f>
         <x:v>46277</x:v>
       </x:c>
-      <x:c r="C8" s="114" t="str">
+      <x:c r="C8" s="143" t="str">
         <x:f>IF(A8="","",'課題入力'!E8)</x:f>
         <x:v>これから</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="112" t="str">
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="141" t="str">
         <x:f>IF('課題入力'!H9=1,'課題入力'!A9,"")</x:f>
       </x:c>
-      <x:c r="B9" s="113" t="str">
+      <x:c r="B9" s="142" t="str">
         <x:f>IF(A9="","",'課題入力'!B9)</x:f>
       </x:c>
-      <x:c r="C9" s="114" t="str">
+      <x:c r="C9" s="143" t="str">
         <x:f>IF(A9="","",'課題入力'!E9)</x:f>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="112" t="str">
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="141" t="str">
         <x:f>IF('課題入力'!H10=1,'課題入力'!A10,"")</x:f>
       </x:c>
-      <x:c r="B10" s="113" t="str">
+      <x:c r="B10" s="142" t="str">
         <x:f>IF(A10="","",'課題入力'!B10)</x:f>
       </x:c>
-      <x:c r="C10" s="114" t="str">
+      <x:c r="C10" s="143" t="str">
         <x:f>IF(A10="","",'課題入力'!E10)</x:f>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="112" t="str">
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="141" t="str">
         <x:f>IF('課題入力'!H11=1,'課題入力'!A11,"")</x:f>
       </x:c>
-      <x:c r="B11" s="113" t="str">
+      <x:c r="B11" s="142" t="str">
         <x:f>IF(A11="","",'課題入力'!B11)</x:f>
       </x:c>
-      <x:c r="C11" s="114" t="str">
+      <x:c r="C11" s="143" t="str">
         <x:f>IF(A11="","",'課題入力'!E11)</x:f>
       </x:c>
     </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="112" t="str">
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="141" t="str">
         <x:f>IF('課題入力'!H12=1,'課題入力'!A12,"")</x:f>
       </x:c>
-      <x:c r="B12" s="113" t="str">
+      <x:c r="B12" s="142" t="str">
         <x:f>IF(A12="","",'課題入力'!B12)</x:f>
       </x:c>
-      <x:c r="C12" s="114" t="str">
+      <x:c r="C12" s="143" t="str">
         <x:f>IF(A12="","",'課題入力'!E12)</x:f>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="112" t="str">
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="141" t="str">
         <x:f>IF('課題入力'!H13=1,'課題入力'!A13,"")</x:f>
       </x:c>
-      <x:c r="B13" s="113" t="str">
+      <x:c r="B13" s="142" t="str">
         <x:f>IF(A13="","",'課題入力'!B13)</x:f>
       </x:c>
-      <x:c r="C13" s="114" t="str">
+      <x:c r="C13" s="143" t="str">
         <x:f>IF(A13="","",'課題入力'!E13)</x:f>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="112" t="str">
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="141" t="str">
         <x:f>IF('課題入力'!H14=1,'課題入力'!A14,"")</x:f>
       </x:c>
-      <x:c r="B14" s="113" t="str">
+      <x:c r="B14" s="142" t="str">
         <x:f>IF(A14="","",'課題入力'!B14)</x:f>
       </x:c>
-      <x:c r="C14" s="114" t="str">
+      <x:c r="C14" s="143" t="str">
         <x:f>IF(A14="","",'課題入力'!E14)</x:f>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="112" t="str">
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="141" t="str">
         <x:f>IF('課題入力'!H15=1,'課題入力'!A15,"")</x:f>
       </x:c>
-      <x:c r="B15" s="113" t="str">
+      <x:c r="B15" s="142" t="str">
         <x:f>IF(A15="","",'課題入力'!B15)</x:f>
       </x:c>
-      <x:c r="C15" s="114" t="str">
+      <x:c r="C15" s="143" t="str">
         <x:f>IF(A15="","",'課題入力'!E15)</x:f>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="112" t="str">
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="141" t="str">
         <x:f>IF('課題入力'!H16=1,'課題入力'!A16,"")</x:f>
       </x:c>
-      <x:c r="B16" s="113" t="str">
+      <x:c r="B16" s="142" t="str">
         <x:f>IF(A16="","",'課題入力'!B16)</x:f>
       </x:c>
-      <x:c r="C16" s="114" t="str">
+      <x:c r="C16" s="143" t="str">
         <x:f>IF(A16="","",'課題入力'!E16)</x:f>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="112" t="str">
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="141" t="str">
         <x:f>IF('課題入力'!H17=1,'課題入力'!A17,"")</x:f>
       </x:c>
-      <x:c r="B17" s="113" t="str">
+      <x:c r="B17" s="142" t="str">
         <x:f>IF(A17="","",'課題入力'!B17)</x:f>
       </x:c>
-      <x:c r="C17" s="114" t="str">
+      <x:c r="C17" s="143" t="str">
         <x:f>IF(A17="","",'課題入力'!E17)</x:f>
       </x:c>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="112" t="str">
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="141" t="str">
         <x:f>IF('課題入力'!H18=1,'課題入力'!A18,"")</x:f>
       </x:c>
-      <x:c r="B18" s="113" t="str">
+      <x:c r="B18" s="142" t="str">
         <x:f>IF(A18="","",'課題入力'!B18)</x:f>
       </x:c>
-      <x:c r="C18" s="114" t="str">
+      <x:c r="C18" s="143" t="str">
         <x:f>IF(A18="","",'課題入力'!E18)</x:f>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="112" t="str">
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="141" t="str">
         <x:f>IF('課題入力'!H19=1,'課題入力'!A19,"")</x:f>
       </x:c>
-      <x:c r="B19" s="113" t="str">
+      <x:c r="B19" s="142" t="str">
         <x:f>IF(A19="","",'課題入力'!B19)</x:f>
       </x:c>
-      <x:c r="C19" s="114" t="str">
+      <x:c r="C19" s="143" t="str">
         <x:f>IF(A19="","",'課題入力'!E19)</x:f>
       </x:c>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="112" t="str">
+    <x:row r="20" ht="24" customHeight="1">
+      <x:c r="A20" s="141" t="str">
         <x:f>IF('課題入力'!H20=1,'課題入力'!A20,"")</x:f>
       </x:c>
-      <x:c r="B20" s="113" t="str">
+      <x:c r="B20" s="142" t="str">
         <x:f>IF(A20="","",'課題入力'!B20)</x:f>
       </x:c>
-      <x:c r="C20" s="114" t="str">
+      <x:c r="C20" s="143" t="str">
         <x:f>IF(A20="","",'課題入力'!E20)</x:f>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="112" t="str">
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="141" t="str">
         <x:f>IF('課題入力'!H21=1,'課題入力'!A21,"")</x:f>
       </x:c>
-      <x:c r="B21" s="113" t="str">
+      <x:c r="B21" s="142" t="str">
         <x:f>IF(A21="","",'課題入力'!B21)</x:f>
       </x:c>
-      <x:c r="C21" s="114" t="str">
+      <x:c r="C21" s="143" t="str">
         <x:f>IF(A21="","",'課題入力'!E21)</x:f>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="112" t="str">
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="141" t="str">
         <x:f>IF('課題入力'!H22=1,'課題入力'!A22,"")</x:f>
       </x:c>
-      <x:c r="B22" s="113" t="str">
+      <x:c r="B22" s="142" t="str">
         <x:f>IF(A22="","",'課題入力'!B22)</x:f>
       </x:c>
-      <x:c r="C22" s="114" t="str">
+      <x:c r="C22" s="143" t="str">
         <x:f>IF(A22="","",'課題入力'!E22)</x:f>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="112" t="str">
+    <x:row r="23" ht="24" customHeight="1">
+      <x:c r="A23" s="141" t="str">
         <x:f>IF('課題入力'!H23=1,'課題入力'!A23,"")</x:f>
       </x:c>
-      <x:c r="B23" s="113" t="str">
+      <x:c r="B23" s="142" t="str">
         <x:f>IF(A23="","",'課題入力'!B23)</x:f>
       </x:c>
-      <x:c r="C23" s="114" t="str">
+      <x:c r="C23" s="143" t="str">
         <x:f>IF(A23="","",'課題入力'!E23)</x:f>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="112" t="str">
+    <x:row r="24" ht="24" customHeight="1">
+      <x:c r="A24" s="141" t="str">
         <x:f>IF('課題入力'!H24=1,'課題入力'!A24,"")</x:f>
       </x:c>
-      <x:c r="B24" s="113" t="str">
+      <x:c r="B24" s="142" t="str">
         <x:f>IF(A24="","",'課題入力'!B24)</x:f>
       </x:c>
-      <x:c r="C24" s="114" t="str">
+      <x:c r="C24" s="143" t="str">
         <x:f>IF(A24="","",'課題入力'!E24)</x:f>
       </x:c>
     </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="112" t="str">
+    <x:row r="25" ht="24" customHeight="1">
+      <x:c r="A25" s="141" t="str">
         <x:f>IF('課題入力'!H25=1,'課題入力'!A25,"")</x:f>
       </x:c>
-      <x:c r="B25" s="113" t="str">
+      <x:c r="B25" s="142" t="str">
         <x:f>IF(A25="","",'課題入力'!B25)</x:f>
       </x:c>
-      <x:c r="C25" s="114" t="str">
+      <x:c r="C25" s="143" t="str">
         <x:f>IF(A25="","",'課題入力'!E25)</x:f>
       </x:c>
     </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="112" t="str">
+    <x:row r="26" ht="24" customHeight="1">
+      <x:c r="A26" s="141" t="str">
         <x:f>IF('課題入力'!H26=1,'課題入力'!A26,"")</x:f>
       </x:c>
-      <x:c r="B26" s="113" t="str">
+      <x:c r="B26" s="142" t="str">
         <x:f>IF(A26="","",'課題入力'!B26)</x:f>
       </x:c>
-      <x:c r="C26" s="114" t="str">
+      <x:c r="C26" s="143" t="str">
         <x:f>IF(A26="","",'課題入力'!E26)</x:f>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="112" t="str">
+    <x:row r="27" ht="24" customHeight="1">
+      <x:c r="A27" s="141" t="str">
         <x:f>IF('課題入力'!H27=1,'課題入力'!A27,"")</x:f>
       </x:c>
-      <x:c r="B27" s="113" t="str">
+      <x:c r="B27" s="142" t="str">
         <x:f>IF(A27="","",'課題入力'!B27)</x:f>
       </x:c>
-      <x:c r="C27" s="114" t="str">
+      <x:c r="C27" s="143" t="str">
         <x:f>IF(A27="","",'課題入力'!E27)</x:f>
       </x:c>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="112" t="str">
+    <x:row r="28" ht="24" customHeight="1">
+      <x:c r="A28" s="141" t="str">
         <x:f>IF('課題入力'!H28=1,'課題入力'!A28,"")</x:f>
       </x:c>
-      <x:c r="B28" s="113" t="str">
+      <x:c r="B28" s="142" t="str">
         <x:f>IF(A28="","",'課題入力'!B28)</x:f>
       </x:c>
-      <x:c r="C28" s="114" t="str">
+      <x:c r="C28" s="143" t="str">
         <x:f>IF(A28="","",'課題入力'!E28)</x:f>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="112" t="str">
+    <x:row r="29" ht="24" customHeight="1">
+      <x:c r="A29" s="141" t="str">
         <x:f>IF('課題入力'!H29=1,'課題入力'!A29,"")</x:f>
       </x:c>
-      <x:c r="B29" s="113" t="str">
+      <x:c r="B29" s="142" t="str">
         <x:f>IF(A29="","",'課題入力'!B29)</x:f>
       </x:c>
-      <x:c r="C29" s="114" t="str">
+      <x:c r="C29" s="143" t="str">
         <x:f>IF(A29="","",'課題入力'!E29)</x:f>
       </x:c>
     </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="112" t="str">
+    <x:row r="30" ht="24" customHeight="1">
+      <x:c r="A30" s="141" t="str">
         <x:f>IF('課題入力'!H30=1,'課題入力'!A30,"")</x:f>
       </x:c>
-      <x:c r="B30" s="113" t="str">
+      <x:c r="B30" s="142" t="str">
         <x:f>IF(A30="","",'課題入力'!B30)</x:f>
       </x:c>
-      <x:c r="C30" s="114" t="str">
+      <x:c r="C30" s="143" t="str">
         <x:f>IF(A30="","",'課題入力'!E30)</x:f>
       </x:c>
     </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="112" t="str">
+    <x:row r="31" ht="24" customHeight="1">
+      <x:c r="A31" s="141" t="str">
         <x:f>IF('課題入力'!H31=1,'課題入力'!A31,"")</x:f>
       </x:c>
-      <x:c r="B31" s="113" t="str">
+      <x:c r="B31" s="142" t="str">
         <x:f>IF(A31="","",'課題入力'!B31)</x:f>
       </x:c>
-      <x:c r="C31" s="114" t="str">
+      <x:c r="C31" s="143" t="str">
         <x:f>IF(A31="","",'課題入力'!E31)</x:f>
       </x:c>
     </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="112" t="str">
+    <x:row r="32" ht="24" customHeight="1">
+      <x:c r="A32" s="141" t="str">
         <x:f>IF('課題入力'!H32=1,'課題入力'!A32,"")</x:f>
       </x:c>
-      <x:c r="B32" s="113" t="str">
+      <x:c r="B32" s="142" t="str">
         <x:f>IF(A32="","",'課題入力'!B32)</x:f>
       </x:c>
-      <x:c r="C32" s="114" t="str">
+      <x:c r="C32" s="143" t="str">
         <x:f>IF(A32="","",'課題入力'!E32)</x:f>
       </x:c>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="112" t="str">
+    <x:row r="33" ht="24" customHeight="1">
+      <x:c r="A33" s="141" t="str">
         <x:f>IF('課題入力'!H33=1,'課題入力'!A33,"")</x:f>
       </x:c>
-      <x:c r="B33" s="113" t="str">
+      <x:c r="B33" s="142" t="str">
         <x:f>IF(A33="","",'課題入力'!B33)</x:f>
       </x:c>
-      <x:c r="C33" s="114" t="str">
+      <x:c r="C33" s="143" t="str">
         <x:f>IF(A33="","",'課題入力'!E33)</x:f>
       </x:c>
     </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="112" t="str">
+    <x:row r="34" ht="24" customHeight="1">
+      <x:c r="A34" s="141" t="str">
         <x:f>IF('課題入力'!H34=1,'課題入力'!A34,"")</x:f>
       </x:c>
-      <x:c r="B34" s="113" t="str">
+      <x:c r="B34" s="142" t="str">
         <x:f>IF(A34="","",'課題入力'!B34)</x:f>
       </x:c>
-      <x:c r="C34" s="114" t="str">
+      <x:c r="C34" s="143" t="str">
         <x:f>IF(A34="","",'課題入力'!E34)</x:f>
       </x:c>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="112" t="str">
+    <x:row r="35" ht="24" customHeight="1">
+      <x:c r="A35" s="141" t="str">
         <x:f>IF('課題入力'!H35=1,'課題入力'!A35,"")</x:f>
       </x:c>
-      <x:c r="B35" s="113" t="str">
+      <x:c r="B35" s="142" t="str">
         <x:f>IF(A35="","",'課題入力'!B35)</x:f>
       </x:c>
-      <x:c r="C35" s="114" t="str">
+      <x:c r="C35" s="143" t="str">
         <x:f>IF(A35="","",'課題入力'!E35)</x:f>
       </x:c>
     </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="112" t="str">
+    <x:row r="36" ht="24" customHeight="1">
+      <x:c r="A36" s="141" t="str">
         <x:f>IF('課題入力'!H36=1,'課題入力'!A36,"")</x:f>
       </x:c>
-      <x:c r="B36" s="113" t="str">
+      <x:c r="B36" s="142" t="str">
         <x:f>IF(A36="","",'課題入力'!B36)</x:f>
       </x:c>
-      <x:c r="C36" s="114" t="str">
+      <x:c r="C36" s="143" t="str">
         <x:f>IF(A36="","",'課題入力'!E36)</x:f>
       </x:c>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="112" t="str">
+    <x:row r="37" ht="24" customHeight="1">
+      <x:c r="A37" s="141" t="str">
         <x:f>IF('課題入力'!H37=1,'課題入力'!A37,"")</x:f>
       </x:c>
-      <x:c r="B37" s="113" t="str">
+      <x:c r="B37" s="142" t="str">
         <x:f>IF(A37="","",'課題入力'!B37)</x:f>
       </x:c>
-      <x:c r="C37" s="114" t="str">
+      <x:c r="C37" s="143" t="str">
         <x:f>IF(A37="","",'課題入力'!E37)</x:f>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="112" t="str">
+    <x:row r="38" ht="24" customHeight="1">
+      <x:c r="A38" s="141" t="str">
         <x:f>IF('課題入力'!H38=1,'課題入力'!A38,"")</x:f>
       </x:c>
-      <x:c r="B38" s="113" t="str">
+      <x:c r="B38" s="142" t="str">
         <x:f>IF(A38="","",'課題入力'!B38)</x:f>
       </x:c>
-      <x:c r="C38" s="114" t="str">
+      <x:c r="C38" s="143" t="str">
         <x:f>IF(A38="","",'課題入力'!E38)</x:f>
       </x:c>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="112" t="str">
+    <x:row r="39" ht="24" customHeight="1">
+      <x:c r="A39" s="141" t="str">
         <x:f>IF('課題入力'!H39=1,'課題入力'!A39,"")</x:f>
       </x:c>
-      <x:c r="B39" s="113" t="str">
+      <x:c r="B39" s="142" t="str">
         <x:f>IF(A39="","",'課題入力'!B39)</x:f>
       </x:c>
-      <x:c r="C39" s="114" t="str">
+      <x:c r="C39" s="143" t="str">
         <x:f>IF(A39="","",'課題入力'!E39)</x:f>
       </x:c>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="112" t="str">
+    <x:row r="40" ht="24" customHeight="1">
+      <x:c r="A40" s="141" t="str">
         <x:f>IF('課題入力'!H40=1,'課題入力'!A40,"")</x:f>
       </x:c>
-      <x:c r="B40" s="113" t="str">
+      <x:c r="B40" s="142" t="str">
         <x:f>IF(A40="","",'課題入力'!B40)</x:f>
       </x:c>
-      <x:c r="C40" s="114" t="str">
+      <x:c r="C40" s="143" t="str">
         <x:f>IF(A40="","",'課題入力'!E40)</x:f>
       </x:c>
     </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="112" t="str">
+    <x:row r="41" ht="24" customHeight="1">
+      <x:c r="A41" s="141" t="str">
         <x:f>IF('課題入力'!H41=1,'課題入力'!A41,"")</x:f>
       </x:c>
-      <x:c r="B41" s="113" t="str">
+      <x:c r="B41" s="142" t="str">
         <x:f>IF(A41="","",'課題入力'!B41)</x:f>
       </x:c>
-      <x:c r="C41" s="114" t="str">
+      <x:c r="C41" s="143" t="str">
         <x:f>IF(A41="","",'課題入力'!E41)</x:f>
       </x:c>
     </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="112" t="str">
+    <x:row r="42" ht="24" customHeight="1">
+      <x:c r="A42" s="141" t="str">
         <x:f>IF('課題入力'!H42=1,'課題入力'!A42,"")</x:f>
       </x:c>
-      <x:c r="B42" s="113" t="str">
+      <x:c r="B42" s="142" t="str">
         <x:f>IF(A42="","",'課題入力'!B42)</x:f>
       </x:c>
-      <x:c r="C42" s="114" t="str">
+      <x:c r="C42" s="143" t="str">
         <x:f>IF(A42="","",'課題入力'!E42)</x:f>
       </x:c>
     </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="112" t="str">
+    <x:row r="43" ht="24" customHeight="1">
+      <x:c r="A43" s="141" t="str">
         <x:f>IF('課題入力'!H43=1,'課題入力'!A43,"")</x:f>
       </x:c>
-      <x:c r="B43" s="113" t="str">
+      <x:c r="B43" s="142" t="str">
         <x:f>IF(A43="","",'課題入力'!B43)</x:f>
       </x:c>
-      <x:c r="C43" s="114" t="str">
+      <x:c r="C43" s="143" t="str">
         <x:f>IF(A43="","",'課題入力'!E43)</x:f>
       </x:c>
     </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="112" t="str">
+    <x:row r="44" ht="24" customHeight="1">
+      <x:c r="A44" s="141" t="str">
         <x:f>IF('課題入力'!H44=1,'課題入力'!A44,"")</x:f>
       </x:c>
-      <x:c r="B44" s="113" t="str">
+      <x:c r="B44" s="142" t="str">
         <x:f>IF(A44="","",'課題入力'!B44)</x:f>
       </x:c>
-      <x:c r="C44" s="114" t="str">
+      <x:c r="C44" s="143" t="str">
         <x:f>IF(A44="","",'課題入力'!E44)</x:f>
       </x:c>
     </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="112" t="str">
+    <x:row r="45" ht="24" customHeight="1">
+      <x:c r="A45" s="141" t="str">
         <x:f>IF('課題入力'!H45=1,'課題入力'!A45,"")</x:f>
       </x:c>
-      <x:c r="B45" s="113" t="str">
+      <x:c r="B45" s="142" t="str">
         <x:f>IF(A45="","",'課題入力'!B45)</x:f>
       </x:c>
-      <x:c r="C45" s="114" t="str">
+      <x:c r="C45" s="143" t="str">
         <x:f>IF(A45="","",'課題入力'!E45)</x:f>
       </x:c>
     </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="112" t="str">
+    <x:row r="46" ht="24" customHeight="1">
+      <x:c r="A46" s="141" t="str">
         <x:f>IF('課題入力'!H46=1,'課題入力'!A46,"")</x:f>
       </x:c>
-      <x:c r="B46" s="113" t="str">
+      <x:c r="B46" s="142" t="str">
         <x:f>IF(A46="","",'課題入力'!B46)</x:f>
       </x:c>
-      <x:c r="C46" s="114" t="str">
+      <x:c r="C46" s="143" t="str">
         <x:f>IF(A46="","",'課題入力'!E46)</x:f>
       </x:c>
     </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="112" t="str">
+    <x:row r="47" ht="24" customHeight="1">
+      <x:c r="A47" s="141" t="str">
         <x:f>IF('課題入力'!H47=1,'課題入力'!A47,"")</x:f>
       </x:c>
-      <x:c r="B47" s="113" t="str">
+      <x:c r="B47" s="142" t="str">
         <x:f>IF(A47="","",'課題入力'!B47)</x:f>
       </x:c>
-      <x:c r="C47" s="114" t="str">
+      <x:c r="C47" s="143" t="str">
         <x:f>IF(A47="","",'課題入力'!E47)</x:f>
       </x:c>
     </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="112" t="str">
+    <x:row r="48" ht="24" customHeight="1">
+      <x:c r="A48" s="141" t="str">
         <x:f>IF('課題入力'!H48=1,'課題入力'!A48,"")</x:f>
       </x:c>
-      <x:c r="B48" s="113" t="str">
+      <x:c r="B48" s="142" t="str">
         <x:f>IF(A48="","",'課題入力'!B48)</x:f>
       </x:c>
-      <x:c r="C48" s="114" t="str">
+      <x:c r="C48" s="143" t="str">
         <x:f>IF(A48="","",'課題入力'!E48)</x:f>
       </x:c>
     </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="112" t="str">
+    <x:row r="49" ht="24" customHeight="1">
+      <x:c r="A49" s="141" t="str">
         <x:f>IF('課題入力'!H49=1,'課題入力'!A49,"")</x:f>
       </x:c>
-      <x:c r="B49" s="113" t="str">
+      <x:c r="B49" s="142" t="str">
         <x:f>IF(A49="","",'課題入力'!B49)</x:f>
       </x:c>
-      <x:c r="C49" s="114" t="str">
+      <x:c r="C49" s="143" t="str">
         <x:f>IF(A49="","",'課題入力'!E49)</x:f>
       </x:c>
     </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="112" t="str">
+    <x:row r="50" ht="24" customHeight="1">
+      <x:c r="A50" s="141" t="str">
         <x:f>IF('課題入力'!H50=1,'課題入力'!A50,"")</x:f>
       </x:c>
-      <x:c r="B50" s="113" t="str">
+      <x:c r="B50" s="142" t="str">
         <x:f>IF(A50="","",'課題入力'!B50)</x:f>
       </x:c>
-      <x:c r="C50" s="114" t="str">
+      <x:c r="C50" s="143" t="str">
         <x:f>IF(A50="","",'課題入力'!E50)</x:f>
       </x:c>
     </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="112" t="str">
+    <x:row r="51" ht="24" customHeight="1">
+      <x:c r="A51" s="141" t="str">
         <x:f>IF('課題入力'!H51=1,'課題入力'!A51,"")</x:f>
       </x:c>
-      <x:c r="B51" s="113" t="str">
+      <x:c r="B51" s="142" t="str">
         <x:f>IF(A51="","",'課題入力'!B51)</x:f>
       </x:c>
-      <x:c r="C51" s="114" t="str">
+      <x:c r="C51" s="143" t="str">
         <x:f>IF(A51="","",'課題入力'!E51)</x:f>
       </x:c>
     </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="112" t="str">
+    <x:row r="52" ht="24" customHeight="1">
+      <x:c r="A52" s="141" t="str">
         <x:f>IF('課題入力'!H52=1,'課題入力'!A52,"")</x:f>
       </x:c>
-      <x:c r="B52" s="113" t="str">
+      <x:c r="B52" s="142" t="str">
         <x:f>IF(A52="","",'課題入力'!B52)</x:f>
       </x:c>
-      <x:c r="C52" s="114" t="str">
+      <x:c r="C52" s="143" t="str">
         <x:f>IF(A52="","",'課題入力'!E52)</x:f>
       </x:c>
     </x:row>
-    <x:row r="53">
-      <x:c r="A53" s="112" t="str">
+    <x:row r="53" ht="24" customHeight="1">
+      <x:c r="A53" s="141" t="str">
         <x:f>IF('課題入力'!H53=1,'課題入力'!A53,"")</x:f>
       </x:c>
-      <x:c r="B53" s="113" t="str">
+      <x:c r="B53" s="142" t="str">
         <x:f>IF(A53="","",'課題入力'!B53)</x:f>
       </x:c>
-      <x:c r="C53" s="114" t="str">
+      <x:c r="C53" s="143" t="str">
         <x:f>IF(A53="","",'課題入力'!E53)</x:f>
       </x:c>
     </x:row>
-    <x:row r="54">
-      <x:c r="A54" s="112" t="str">
+    <x:row r="54" ht="24" customHeight="1">
+      <x:c r="A54" s="141" t="str">
         <x:f>IF('課題入力'!H54=1,'課題入力'!A54,"")</x:f>
       </x:c>
-      <x:c r="B54" s="113" t="str">
+      <x:c r="B54" s="142" t="str">
         <x:f>IF(A54="","",'課題入力'!B54)</x:f>
       </x:c>
-      <x:c r="C54" s="114" t="str">
+      <x:c r="C54" s="143" t="str">
         <x:f>IF(A54="","",'課題入力'!E54)</x:f>
       </x:c>
     </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="112" t="str">
+    <x:row r="55" ht="24" customHeight="1">
+      <x:c r="A55" s="141" t="str">
         <x:f>IF('課題入力'!H55=1,'課題入力'!A55,"")</x:f>
       </x:c>
-      <x:c r="B55" s="113" t="str">
+      <x:c r="B55" s="142" t="str">
         <x:f>IF(A55="","",'課題入力'!B55)</x:f>
       </x:c>
-      <x:c r="C55" s="114" t="str">
+      <x:c r="C55" s="143" t="str">
         <x:f>IF(A55="","",'課題入力'!E55)</x:f>
       </x:c>
     </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="112" t="str">
+    <x:row r="56" ht="24" customHeight="1">
+      <x:c r="A56" s="141" t="str">
         <x:f>IF('課題入力'!H56=1,'課題入力'!A56,"")</x:f>
       </x:c>
-      <x:c r="B56" s="113" t="str">
+      <x:c r="B56" s="142" t="str">
         <x:f>IF(A56="","",'課題入力'!B56)</x:f>
       </x:c>
-      <x:c r="C56" s="114" t="str">
+      <x:c r="C56" s="143" t="str">
         <x:f>IF(A56="","",'課題入力'!E56)</x:f>
       </x:c>
     </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="112" t="str">
+    <x:row r="57" ht="24" customHeight="1">
+      <x:c r="A57" s="141" t="str">
         <x:f>IF('課題入力'!H57=1,'課題入力'!A57,"")</x:f>
       </x:c>
-      <x:c r="B57" s="113" t="str">
+      <x:c r="B57" s="142" t="str">
         <x:f>IF(A57="","",'課題入力'!B57)</x:f>
       </x:c>
-      <x:c r="C57" s="114" t="str">
+      <x:c r="C57" s="143" t="str">
         <x:f>IF(A57="","",'課題入力'!E57)</x:f>
       </x:c>
     </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="112" t="str">
+    <x:row r="58" ht="24" customHeight="1">
+      <x:c r="A58" s="141" t="str">
         <x:f>IF('課題入力'!H58=1,'課題入力'!A58,"")</x:f>
       </x:c>
-      <x:c r="B58" s="113" t="str">
+      <x:c r="B58" s="142" t="str">
         <x:f>IF(A58="","",'課題入力'!B58)</x:f>
       </x:c>
-      <x:c r="C58" s="114" t="str">
+      <x:c r="C58" s="143" t="str">
         <x:f>IF(A58="","",'課題入力'!E58)</x:f>
       </x:c>
     </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="112" t="str">
+    <x:row r="59" ht="24" customHeight="1">
+      <x:c r="A59" s="141" t="str">
         <x:f>IF('課題入力'!H59=1,'課題入力'!A59,"")</x:f>
       </x:c>
-      <x:c r="B59" s="113" t="str">
+      <x:c r="B59" s="142" t="str">
         <x:f>IF(A59="","",'課題入力'!B59)</x:f>
       </x:c>
-      <x:c r="C59" s="114" t="str">
+      <x:c r="C59" s="143" t="str">
         <x:f>IF(A59="","",'課題入力'!E59)</x:f>
       </x:c>
     </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="112" t="str">
+    <x:row r="60" ht="24" customHeight="1">
+      <x:c r="A60" s="141" t="str">
         <x:f>IF('課題入力'!H60=1,'課題入力'!A60,"")</x:f>
       </x:c>
-      <x:c r="B60" s="113" t="str">
+      <x:c r="B60" s="142" t="str">
         <x:f>IF(A60="","",'課題入力'!B60)</x:f>
       </x:c>
-      <x:c r="C60" s="114" t="str">
+      <x:c r="C60" s="143" t="str">
         <x:f>IF(A60="","",'課題入力'!E60)</x:f>
       </x:c>
     </x:row>
-    <x:row r="61">
-      <x:c r="A61" s="112" t="str">
+    <x:row r="61" ht="24" customHeight="1">
+      <x:c r="A61" s="141" t="str">
         <x:f>IF('課題入力'!H61=1,'課題入力'!A61,"")</x:f>
       </x:c>
-      <x:c r="B61" s="113" t="str">
+      <x:c r="B61" s="142" t="str">
         <x:f>IF(A61="","",'課題入力'!B61)</x:f>
       </x:c>
-      <x:c r="C61" s="114" t="str">
+      <x:c r="C61" s="143" t="str">
         <x:f>IF(A61="","",'課題入力'!E61)</x:f>
       </x:c>
     </x:row>
-    <x:row r="62">
-      <x:c r="A62" s="112" t="str">
+    <x:row r="62" ht="24" customHeight="1">
+      <x:c r="A62" s="141" t="str">
         <x:f>IF('課題入力'!H62=1,'課題入力'!A62,"")</x:f>
       </x:c>
-      <x:c r="B62" s="113" t="str">
+      <x:c r="B62" s="142" t="str">
         <x:f>IF(A62="","",'課題入力'!B62)</x:f>
       </x:c>
-      <x:c r="C62" s="114" t="str">
+      <x:c r="C62" s="143" t="str">
         <x:f>IF(A62="","",'課題入力'!E62)</x:f>
       </x:c>
     </x:row>
-    <x:row r="63">
-      <x:c r="A63" s="112" t="str">
+    <x:row r="63" ht="24" customHeight="1">
+      <x:c r="A63" s="141" t="str">
         <x:f>IF('課題入力'!H63=1,'課題入力'!A63,"")</x:f>
       </x:c>
-      <x:c r="B63" s="113" t="str">
+      <x:c r="B63" s="142" t="str">
         <x:f>IF(A63="","",'課題入力'!B63)</x:f>
       </x:c>
-      <x:c r="C63" s="114" t="str">
+      <x:c r="C63" s="143" t="str">
         <x:f>IF(A63="","",'課題入力'!E63)</x:f>
       </x:c>
     </x:row>
-    <x:row r="64">
-      <x:c r="A64" s="112" t="str">
+    <x:row r="64" ht="24" customHeight="1">
+      <x:c r="A64" s="141" t="str">
         <x:f>IF('課題入力'!H64=1,'課題入力'!A64,"")</x:f>
       </x:c>
-      <x:c r="B64" s="113" t="str">
+      <x:c r="B64" s="142" t="str">
         <x:f>IF(A64="","",'課題入力'!B64)</x:f>
       </x:c>
-      <x:c r="C64" s="114" t="str">
+      <x:c r="C64" s="143" t="str">
         <x:f>IF(A64="","",'課題入力'!E64)</x:f>
       </x:c>
     </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="112" t="str">
+    <x:row r="65" ht="24" customHeight="1">
+      <x:c r="A65" s="141" t="str">
         <x:f>IF('課題入力'!H65=1,'課題入力'!A65,"")</x:f>
       </x:c>
-      <x:c r="B65" s="113" t="str">
+      <x:c r="B65" s="142" t="str">
         <x:f>IF(A65="","",'課題入力'!B65)</x:f>
       </x:c>
-      <x:c r="C65" s="114" t="str">
+      <x:c r="C65" s="143" t="str">
         <x:f>IF(A65="","",'課題入力'!E65)</x:f>
       </x:c>
     </x:row>
-    <x:row r="66">
-      <x:c r="A66" s="112" t="str">
+    <x:row r="66" ht="24" customHeight="1">
+      <x:c r="A66" s="141" t="str">
         <x:f>IF('課題入力'!H66=1,'課題入力'!A66,"")</x:f>
       </x:c>
-      <x:c r="B66" s="113" t="str">
+      <x:c r="B66" s="142" t="str">
         <x:f>IF(A66="","",'課題入力'!B66)</x:f>
       </x:c>
-      <x:c r="C66" s="114" t="str">
+      <x:c r="C66" s="143" t="str">
         <x:f>IF(A66="","",'課題入力'!E66)</x:f>
       </x:c>
     </x:row>
-    <x:row r="67">
-      <x:c r="A67" s="112" t="str">
+    <x:row r="67" ht="24" customHeight="1">
+      <x:c r="A67" s="141" t="str">
         <x:f>IF('課題入力'!H67=1,'課題入力'!A67,"")</x:f>
       </x:c>
-      <x:c r="B67" s="113" t="str">
+      <x:c r="B67" s="142" t="str">
         <x:f>IF(A67="","",'課題入力'!B67)</x:f>
       </x:c>
-      <x:c r="C67" s="114" t="str">
+      <x:c r="C67" s="143" t="str">
         <x:f>IF(A67="","",'課題入力'!E67)</x:f>
       </x:c>
     </x:row>
-    <x:row r="68">
-      <x:c r="A68" s="112" t="str">
+    <x:row r="68" ht="24" customHeight="1">
+      <x:c r="A68" s="141" t="str">
         <x:f>IF('課題入力'!H68=1,'課題入力'!A68,"")</x:f>
       </x:c>
-      <x:c r="B68" s="113" t="str">
+      <x:c r="B68" s="142" t="str">
         <x:f>IF(A68="","",'課題入力'!B68)</x:f>
       </x:c>
-      <x:c r="C68" s="114" t="str">
+      <x:c r="C68" s="143" t="str">
         <x:f>IF(A68="","",'課題入力'!E68)</x:f>
       </x:c>
     </x:row>
-    <x:row r="69">
-      <x:c r="A69" s="112" t="str">
+    <x:row r="69" ht="24" customHeight="1">
+      <x:c r="A69" s="141" t="str">
         <x:f>IF('課題入力'!H69=1,'課題入力'!A69,"")</x:f>
       </x:c>
-      <x:c r="B69" s="113" t="str">
+      <x:c r="B69" s="142" t="str">
         <x:f>IF(A69="","",'課題入力'!B69)</x:f>
       </x:c>
-      <x:c r="C69" s="114" t="str">
+      <x:c r="C69" s="143" t="str">
         <x:f>IF(A69="","",'課題入力'!E69)</x:f>
       </x:c>
     </x:row>
-    <x:row r="70">
-      <x:c r="A70" s="112" t="str">
+    <x:row r="70" ht="24" customHeight="1">
+      <x:c r="A70" s="141" t="str">
         <x:f>IF('課題入力'!H70=1,'課題入力'!A70,"")</x:f>
       </x:c>
-      <x:c r="B70" s="113" t="str">
+      <x:c r="B70" s="142" t="str">
         <x:f>IF(A70="","",'課題入力'!B70)</x:f>
       </x:c>
-      <x:c r="C70" s="114" t="str">
+      <x:c r="C70" s="143" t="str">
         <x:f>IF(A70="","",'課題入力'!E70)</x:f>
       </x:c>
     </x:row>
-    <x:row r="71">
-      <x:c r="A71" s="112" t="str">
+    <x:row r="71" ht="24" customHeight="1">
+      <x:c r="A71" s="141" t="str">
         <x:f>IF('課題入力'!H71=1,'課題入力'!A71,"")</x:f>
       </x:c>
-      <x:c r="B71" s="113" t="str">
+      <x:c r="B71" s="142" t="str">
         <x:f>IF(A71="","",'課題入力'!B71)</x:f>
       </x:c>
-      <x:c r="C71" s="114" t="str">
+      <x:c r="C71" s="143" t="str">
         <x:f>IF(A71="","",'課題入力'!E71)</x:f>
       </x:c>
     </x:row>
-    <x:row r="72">
-      <x:c r="A72" s="112" t="str">
+    <x:row r="72" ht="24" customHeight="1">
+      <x:c r="A72" s="141" t="str">
         <x:f>IF('課題入力'!H72=1,'課題入力'!A72,"")</x:f>
       </x:c>
-      <x:c r="B72" s="113" t="str">
+      <x:c r="B72" s="142" t="str">
         <x:f>IF(A72="","",'課題入力'!B72)</x:f>
       </x:c>
-      <x:c r="C72" s="114" t="str">
+      <x:c r="C72" s="143" t="str">
         <x:f>IF(A72="","",'課題入力'!E72)</x:f>
       </x:c>
     </x:row>
-    <x:row r="73">
-      <x:c r="A73" s="112" t="str">
+    <x:row r="73" ht="24" customHeight="1">
+      <x:c r="A73" s="141" t="str">
         <x:f>IF('課題入力'!H73=1,'課題入力'!A73,"")</x:f>
       </x:c>
-      <x:c r="B73" s="113" t="str">
+      <x:c r="B73" s="142" t="str">
         <x:f>IF(A73="","",'課題入力'!B73)</x:f>
       </x:c>
-      <x:c r="C73" s="114" t="str">
+      <x:c r="C73" s="143" t="str">
         <x:f>IF(A73="","",'課題入力'!E73)</x:f>
       </x:c>
     </x:row>
-    <x:row r="74">
-      <x:c r="A74" s="112" t="str">
+    <x:row r="74" ht="24" customHeight="1">
+      <x:c r="A74" s="141" t="str">
         <x:f>IF('課題入力'!H74=1,'課題入力'!A74,"")</x:f>
       </x:c>
-      <x:c r="B74" s="113" t="str">
+      <x:c r="B74" s="142" t="str">
         <x:f>IF(A74="","",'課題入力'!B74)</x:f>
       </x:c>
-      <x:c r="C74" s="114" t="str">
+      <x:c r="C74" s="143" t="str">
         <x:f>IF(A74="","",'課題入力'!E74)</x:f>
       </x:c>
     </x:row>
-    <x:row r="75">
-      <x:c r="A75" s="112" t="str">
+    <x:row r="75" ht="24" customHeight="1">
+      <x:c r="A75" s="141" t="str">
         <x:f>IF('課題入力'!H75=1,'課題入力'!A75,"")</x:f>
       </x:c>
-      <x:c r="B75" s="113" t="str">
+      <x:c r="B75" s="142" t="str">
         <x:f>IF(A75="","",'課題入力'!B75)</x:f>
       </x:c>
-      <x:c r="C75" s="114" t="str">
+      <x:c r="C75" s="143" t="str">
         <x:f>IF(A75="","",'課題入力'!E75)</x:f>
       </x:c>
     </x:row>
-    <x:row r="76">
-      <x:c r="A76" s="112" t="str">
+    <x:row r="76" ht="24" customHeight="1">
+      <x:c r="A76" s="141" t="str">
         <x:f>IF('課題入力'!H76=1,'課題入力'!A76,"")</x:f>
       </x:c>
-      <x:c r="B76" s="113" t="str">
+      <x:c r="B76" s="142" t="str">
         <x:f>IF(A76="","",'課題入力'!B76)</x:f>
       </x:c>
-      <x:c r="C76" s="114" t="str">
+      <x:c r="C76" s="143" t="str">
         <x:f>IF(A76="","",'課題入力'!E76)</x:f>
       </x:c>
     </x:row>
-    <x:row r="77">
-      <x:c r="A77" s="112" t="str">
+    <x:row r="77" ht="24" customHeight="1">
+      <x:c r="A77" s="141" t="str">
         <x:f>IF('課題入力'!H77=1,'課題入力'!A77,"")</x:f>
       </x:c>
-      <x:c r="B77" s="113" t="str">
+      <x:c r="B77" s="142" t="str">
         <x:f>IF(A77="","",'課題入力'!B77)</x:f>
       </x:c>
-      <x:c r="C77" s="114" t="str">
+      <x:c r="C77" s="143" t="str">
         <x:f>IF(A77="","",'課題入力'!E77)</x:f>
       </x:c>
     </x:row>
-    <x:row r="78">
-      <x:c r="A78" s="112" t="str">
+    <x:row r="78" ht="24" customHeight="1">
+      <x:c r="A78" s="141" t="str">
         <x:f>IF('課題入力'!H78=1,'課題入力'!A78,"")</x:f>
       </x:c>
-      <x:c r="B78" s="113" t="str">
+      <x:c r="B78" s="142" t="str">
         <x:f>IF(A78="","",'課題入力'!B78)</x:f>
       </x:c>
-      <x:c r="C78" s="114" t="str">
+      <x:c r="C78" s="143" t="str">
         <x:f>IF(A78="","",'課題入力'!E78)</x:f>
       </x:c>
     </x:row>
-    <x:row r="79">
-      <x:c r="A79" s="112" t="str">
+    <x:row r="79" ht="24" customHeight="1">
+      <x:c r="A79" s="141" t="str">
         <x:f>IF('課題入力'!H79=1,'課題入力'!A79,"")</x:f>
       </x:c>
-      <x:c r="B79" s="113" t="str">
+      <x:c r="B79" s="142" t="str">
         <x:f>IF(A79="","",'課題入力'!B79)</x:f>
       </x:c>
-      <x:c r="C79" s="114" t="str">
+      <x:c r="C79" s="143" t="str">
         <x:f>IF(A79="","",'課題入力'!E79)</x:f>
       </x:c>
     </x:row>
-    <x:row r="80">
-      <x:c r="A80" s="112" t="str">
+    <x:row r="80" ht="24" customHeight="1">
+      <x:c r="A80" s="141" t="str">
         <x:f>IF('課題入力'!H80=1,'課題入力'!A80,"")</x:f>
       </x:c>
-      <x:c r="B80" s="113" t="str">
+      <x:c r="B80" s="142" t="str">
         <x:f>IF(A80="","",'課題入力'!B80)</x:f>
       </x:c>
-      <x:c r="C80" s="114" t="str">
+      <x:c r="C80" s="143" t="str">
         <x:f>IF(A80="","",'課題入力'!E80)</x:f>
       </x:c>
     </x:row>
-    <x:row r="81">
-      <x:c r="A81" s="112" t="str">
+    <x:row r="81" ht="24" customHeight="1">
+      <x:c r="A81" s="141" t="str">
         <x:f>IF('課題入力'!H81=1,'課題入力'!A81,"")</x:f>
       </x:c>
-      <x:c r="B81" s="113" t="str">
+      <x:c r="B81" s="142" t="str">
         <x:f>IF(A81="","",'課題入力'!B81)</x:f>
       </x:c>
-      <x:c r="C81" s="114" t="str">
+      <x:c r="C81" s="143" t="str">
         <x:f>IF(A81="","",'課題入力'!E81)</x:f>
       </x:c>
     </x:row>
-    <x:row r="82">
-      <x:c r="A82" s="112" t="str">
+    <x:row r="82" ht="24" customHeight="1">
+      <x:c r="A82" s="141" t="str">
         <x:f>IF('課題入力'!H82=1,'課題入力'!A82,"")</x:f>
       </x:c>
-      <x:c r="B82" s="113" t="str">
+      <x:c r="B82" s="142" t="str">
         <x:f>IF(A82="","",'課題入力'!B82)</x:f>
       </x:c>
-      <x:c r="C82" s="114" t="str">
+      <x:c r="C82" s="143" t="str">
         <x:f>IF(A82="","",'課題入力'!E82)</x:f>
       </x:c>
     </x:row>
-    <x:row r="83">
-      <x:c r="A83" s="112" t="str">
+    <x:row r="83" ht="24" customHeight="1">
+      <x:c r="A83" s="141" t="str">
         <x:f>IF('課題入力'!H83=1,'課題入力'!A83,"")</x:f>
       </x:c>
-      <x:c r="B83" s="113" t="str">
+      <x:c r="B83" s="142" t="str">
         <x:f>IF(A83="","",'課題入力'!B83)</x:f>
       </x:c>
-      <x:c r="C83" s="114" t="str">
+      <x:c r="C83" s="143" t="str">
         <x:f>IF(A83="","",'課題入力'!E83)</x:f>
       </x:c>
     </x:row>
-    <x:row r="84">
-      <x:c r="A84" s="112" t="str">
+    <x:row r="84" ht="24" customHeight="1">
+      <x:c r="A84" s="141" t="str">
         <x:f>IF('課題入力'!H84=1,'課題入力'!A84,"")</x:f>
       </x:c>
-      <x:c r="B84" s="113" t="str">
+      <x:c r="B84" s="142" t="str">
         <x:f>IF(A84="","",'課題入力'!B84)</x:f>
       </x:c>
-      <x:c r="C84" s="114" t="str">
+      <x:c r="C84" s="143" t="str">
         <x:f>IF(A84="","",'課題入力'!E84)</x:f>
       </x:c>
     </x:row>
-    <x:row r="85">
-      <x:c r="A85" s="112" t="str">
+    <x:row r="85" ht="24" customHeight="1">
+      <x:c r="A85" s="141" t="str">
         <x:f>IF('課題入力'!H85=1,'課題入力'!A85,"")</x:f>
       </x:c>
-      <x:c r="B85" s="113" t="str">
+      <x:c r="B85" s="142" t="str">
         <x:f>IF(A85="","",'課題入力'!B85)</x:f>
       </x:c>
-      <x:c r="C85" s="114" t="str">
+      <x:c r="C85" s="143" t="str">
         <x:f>IF(A85="","",'課題入力'!E85)</x:f>
       </x:c>
     </x:row>
-    <x:row r="86">
-      <x:c r="A86" s="112" t="str">
+    <x:row r="86" ht="24" customHeight="1">
+      <x:c r="A86" s="141" t="str">
         <x:f>IF('課題入力'!H86=1,'課題入力'!A86,"")</x:f>
       </x:c>
-      <x:c r="B86" s="113" t="str">
+      <x:c r="B86" s="142" t="str">
         <x:f>IF(A86="","",'課題入力'!B86)</x:f>
       </x:c>
-      <x:c r="C86" s="114" t="str">
+      <x:c r="C86" s="143" t="str">
         <x:f>IF(A86="","",'課題入力'!E86)</x:f>
       </x:c>
     </x:row>
-    <x:row r="87">
-      <x:c r="A87" s="112" t="str">
+    <x:row r="87" ht="24" customHeight="1">
+      <x:c r="A87" s="141" t="str">
         <x:f>IF('課題入力'!H87=1,'課題入力'!A87,"")</x:f>
       </x:c>
-      <x:c r="B87" s="113" t="str">
+      <x:c r="B87" s="142" t="str">
         <x:f>IF(A87="","",'課題入力'!B87)</x:f>
       </x:c>
-      <x:c r="C87" s="114" t="str">
+      <x:c r="C87" s="143" t="str">
         <x:f>IF(A87="","",'課題入力'!E87)</x:f>
       </x:c>
     </x:row>
-    <x:row r="88">
-      <x:c r="A88" s="112" t="str">
+    <x:row r="88" ht="24" customHeight="1">
+      <x:c r="A88" s="141" t="str">
         <x:f>IF('課題入力'!H88=1,'課題入力'!A88,"")</x:f>
       </x:c>
-      <x:c r="B88" s="113" t="str">
+      <x:c r="B88" s="142" t="str">
         <x:f>IF(A88="","",'課題入力'!B88)</x:f>
       </x:c>
-      <x:c r="C88" s="114" t="str">
+      <x:c r="C88" s="143" t="str">
         <x:f>IF(A88="","",'課題入力'!E88)</x:f>
       </x:c>
     </x:row>
-    <x:row r="89">
-      <x:c r="A89" s="112" t="str">
+    <x:row r="89" ht="24" customHeight="1">
+      <x:c r="A89" s="141" t="str">
         <x:f>IF('課題入力'!H89=1,'課題入力'!A89,"")</x:f>
       </x:c>
-      <x:c r="B89" s="113" t="str">
+      <x:c r="B89" s="142" t="str">
         <x:f>IF(A89="","",'課題入力'!B89)</x:f>
       </x:c>
-      <x:c r="C89" s="114" t="str">
+      <x:c r="C89" s="143" t="str">
         <x:f>IF(A89="","",'課題入力'!E89)</x:f>
       </x:c>
     </x:row>
-    <x:row r="90">
-      <x:c r="A90" s="112" t="str">
+    <x:row r="90" ht="24" customHeight="1">
+      <x:c r="A90" s="141" t="str">
         <x:f>IF('課題入力'!H90=1,'課題入力'!A90,"")</x:f>
       </x:c>
-      <x:c r="B90" s="113" t="str">
+      <x:c r="B90" s="142" t="str">
         <x:f>IF(A90="","",'課題入力'!B90)</x:f>
       </x:c>
-      <x:c r="C90" s="114" t="str">
+      <x:c r="C90" s="143" t="str">
         <x:f>IF(A90="","",'課題入力'!E90)</x:f>
       </x:c>
     </x:row>
-    <x:row r="91">
-      <x:c r="A91" s="112" t="str">
+    <x:row r="91" ht="24" customHeight="1">
+      <x:c r="A91" s="141" t="str">
         <x:f>IF('課題入力'!H91=1,'課題入力'!A91,"")</x:f>
       </x:c>
-      <x:c r="B91" s="113" t="str">
+      <x:c r="B91" s="142" t="str">
         <x:f>IF(A91="","",'課題入力'!B91)</x:f>
       </x:c>
-      <x:c r="C91" s="114" t="str">
+      <x:c r="C91" s="143" t="str">
         <x:f>IF(A91="","",'課題入力'!E91)</x:f>
       </x:c>
     </x:row>
-    <x:row r="92">
-      <x:c r="A92" s="112" t="str">
+    <x:row r="92" ht="24" customHeight="1">
+      <x:c r="A92" s="141" t="str">
         <x:f>IF('課題入力'!H92=1,'課題入力'!A92,"")</x:f>
       </x:c>
-      <x:c r="B92" s="113" t="str">
+      <x:c r="B92" s="142" t="str">
         <x:f>IF(A92="","",'課題入力'!B92)</x:f>
       </x:c>
-      <x:c r="C92" s="114" t="str">
+      <x:c r="C92" s="143" t="str">
         <x:f>IF(A92="","",'課題入力'!E92)</x:f>
       </x:c>
     </x:row>
-    <x:row r="93">
-      <x:c r="A93" s="112" t="str">
+    <x:row r="93" ht="24" customHeight="1">
+      <x:c r="A93" s="141" t="str">
         <x:f>IF('課題入力'!H93=1,'課題入力'!A93,"")</x:f>
       </x:c>
-      <x:c r="B93" s="113" t="str">
+      <x:c r="B93" s="142" t="str">
         <x:f>IF(A93="","",'課題入力'!B93)</x:f>
       </x:c>
-      <x:c r="C93" s="114" t="str">
+      <x:c r="C93" s="143" t="str">
         <x:f>IF(A93="","",'課題入力'!E93)</x:f>
       </x:c>
     </x:row>
-    <x:row r="94">
-      <x:c r="A94" s="112" t="str">
+    <x:row r="94" ht="24" customHeight="1">
+      <x:c r="A94" s="141" t="str">
         <x:f>IF('課題入力'!H94=1,'課題入力'!A94,"")</x:f>
       </x:c>
-      <x:c r="B94" s="113" t="str">
+      <x:c r="B94" s="142" t="str">
         <x:f>IF(A94="","",'課題入力'!B94)</x:f>
       </x:c>
-      <x:c r="C94" s="114" t="str">
+      <x:c r="C94" s="143" t="str">
         <x:f>IF(A94="","",'課題入力'!E94)</x:f>
       </x:c>
     </x:row>
-    <x:row r="95">
-      <x:c r="A95" s="112" t="str">
+    <x:row r="95" ht="24" customHeight="1">
+      <x:c r="A95" s="141" t="str">
         <x:f>IF('課題入力'!H95=1,'課題入力'!A95,"")</x:f>
       </x:c>
-      <x:c r="B95" s="113" t="str">
+      <x:c r="B95" s="142" t="str">
         <x:f>IF(A95="","",'課題入力'!B95)</x:f>
       </x:c>
-      <x:c r="C95" s="114" t="str">
+      <x:c r="C95" s="143" t="str">
         <x:f>IF(A95="","",'課題入力'!E95)</x:f>
       </x:c>
     </x:row>
-    <x:row r="96">
-      <x:c r="A96" s="112" t="str">
+    <x:row r="96" ht="24" customHeight="1">
+      <x:c r="A96" s="141" t="str">
         <x:f>IF('課題入力'!H96=1,'課題入力'!A96,"")</x:f>
       </x:c>
-      <x:c r="B96" s="113" t="str">
+      <x:c r="B96" s="142" t="str">
         <x:f>IF(A96="","",'課題入力'!B96)</x:f>
       </x:c>
-      <x:c r="C96" s="114" t="str">
+      <x:c r="C96" s="143" t="str">
         <x:f>IF(A96="","",'課題入力'!E96)</x:f>
       </x:c>
     </x:row>
-    <x:row r="97">
-      <x:c r="A97" s="112" t="str">
+    <x:row r="97" ht="24" customHeight="1">
+      <x:c r="A97" s="141" t="str">
         <x:f>IF('課題入力'!H97=1,'課題入力'!A97,"")</x:f>
       </x:c>
-      <x:c r="B97" s="113" t="str">
+      <x:c r="B97" s="142" t="str">
         <x:f>IF(A97="","",'課題入力'!B97)</x:f>
       </x:c>
-      <x:c r="C97" s="114" t="str">
+      <x:c r="C97" s="143" t="str">
         <x:f>IF(A97="","",'課題入力'!E97)</x:f>
       </x:c>
     </x:row>
-    <x:row r="98">
-      <x:c r="A98" s="112" t="str">
+    <x:row r="98" ht="24" customHeight="1">
+      <x:c r="A98" s="141" t="str">
         <x:f>IF('課題入力'!H98=1,'課題入力'!A98,"")</x:f>
       </x:c>
-      <x:c r="B98" s="113" t="str">
+      <x:c r="B98" s="142" t="str">
         <x:f>IF(A98="","",'課題入力'!B98)</x:f>
       </x:c>
-      <x:c r="C98" s="114" t="str">
+      <x:c r="C98" s="143" t="str">
         <x:f>IF(A98="","",'課題入力'!E98)</x:f>
       </x:c>
     </x:row>
-    <x:row r="99">
-      <x:c r="A99" s="112" t="str">
+    <x:row r="99" ht="24" customHeight="1">
+      <x:c r="A99" s="141" t="str">
         <x:f>IF('課題入力'!H99=1,'課題入力'!A99,"")</x:f>
       </x:c>
-      <x:c r="B99" s="113" t="str">
+      <x:c r="B99" s="142" t="str">
         <x:f>IF(A99="","",'課題入力'!B99)</x:f>
       </x:c>
-      <x:c r="C99" s="114" t="str">
+      <x:c r="C99" s="143" t="str">
         <x:f>IF(A99="","",'課題入力'!E99)</x:f>
       </x:c>
     </x:row>
-    <x:row r="100">
-      <x:c r="A100" s="112" t="str">
+    <x:row r="100" ht="24" customHeight="1">
+      <x:c r="A100" s="141" t="str">
         <x:f>IF('課題入力'!H100=1,'課題入力'!A100,"")</x:f>
       </x:c>
-      <x:c r="B100" s="113" t="str">
+      <x:c r="B100" s="142" t="str">
         <x:f>IF(A100="","",'課題入力'!B100)</x:f>
       </x:c>
-      <x:c r="C100" s="114" t="str">
+      <x:c r="C100" s="143" t="str">
         <x:f>IF(A100="","",'課題入力'!E100)</x:f>
       </x:c>
     </x:row>
-    <x:row r="101">
-      <x:c r="A101" s="112" t="str">
+    <x:row r="101" ht="24" customHeight="1">
+      <x:c r="A101" s="141" t="str">
         <x:f>IF('課題入力'!H101=1,'課題入力'!A101,"")</x:f>
       </x:c>
-      <x:c r="B101" s="113" t="str">
+      <x:c r="B101" s="142" t="str">
         <x:f>IF(A101="","",'課題入力'!B101)</x:f>
       </x:c>
-      <x:c r="C101" s="114" t="str">
+      <x:c r="C101" s="143" t="str">
         <x:f>IF(A101="","",'課題入力'!E101)</x:f>
       </x:c>
     </x:row>
-    <x:row r="102">
-      <x:c r="A102" s="112" t="str">
+    <x:row r="102" ht="24" customHeight="1">
+      <x:c r="A102" s="141" t="str">
         <x:f>IF('課題入力'!H102=1,'課題入力'!A102,"")</x:f>
       </x:c>
-      <x:c r="B102" s="113" t="str">
+      <x:c r="B102" s="142" t="str">
         <x:f>IF(A102="","",'課題入力'!B102)</x:f>
       </x:c>
-      <x:c r="C102" s="114" t="str">
+      <x:c r="C102" s="143" t="str">
         <x:f>IF(A102="","",'課題入力'!E102)</x:f>
       </x:c>
     </x:row>
-    <x:row r="103">
-      <x:c r="A103" s="112" t="str">
+    <x:row r="103" ht="24" customHeight="1">
+      <x:c r="A103" s="141" t="str">
         <x:f>IF('課題入力'!H103=1,'課題入力'!A103,"")</x:f>
       </x:c>
-      <x:c r="B103" s="113" t="str">
+      <x:c r="B103" s="142" t="str">
         <x:f>IF(A103="","",'課題入力'!B103)</x:f>
       </x:c>
-      <x:c r="C103" s="114" t="str">
+      <x:c r="C103" s="143" t="str">
         <x:f>IF(A103="","",'課題入力'!E103)</x:f>
       </x:c>
     </x:row>
-    <x:row r="104">
-      <x:c r="A104" s="112" t="str">
+    <x:row r="104" ht="24" customHeight="1">
+      <x:c r="A104" s="141" t="str">
         <x:f>IF('課題入力'!H104=1,'課題入力'!A104,"")</x:f>
       </x:c>
-      <x:c r="B104" s="113" t="str">
+      <x:c r="B104" s="142" t="str">
         <x:f>IF(A104="","",'課題入力'!B104)</x:f>
       </x:c>
-      <x:c r="C104" s="114" t="str">
+      <x:c r="C104" s="143" t="str">
         <x:f>IF(A104="","",'課題入力'!E104)</x:f>
       </x:c>
     </x:row>
-    <x:row r="105">
-      <x:c r="A105" s="112" t="str">
+    <x:row r="105" ht="24" customHeight="1">
+      <x:c r="A105" s="141" t="str">
         <x:f>IF('課題入力'!H105=1,'課題入力'!A105,"")</x:f>
       </x:c>
-      <x:c r="B105" s="113" t="str">
+      <x:c r="B105" s="142" t="str">
         <x:f>IF(A105="","",'課題入力'!B105)</x:f>
       </x:c>
-      <x:c r="C105" s="114" t="str">
+      <x:c r="C105" s="143" t="str">
         <x:f>IF(A105="","",'課題入力'!E105)</x:f>
       </x:c>
     </x:row>
-    <x:row r="106">
-      <x:c r="A106" s="112" t="str">
+    <x:row r="106" ht="24" customHeight="1">
+      <x:c r="A106" s="141" t="str">
         <x:f>IF('課題入力'!H106=1,'課題入力'!A106,"")</x:f>
       </x:c>
-      <x:c r="B106" s="113" t="str">
+      <x:c r="B106" s="142" t="str">
         <x:f>IF(A106="","",'課題入力'!B106)</x:f>
       </x:c>
-      <x:c r="C106" s="114" t="str">
+      <x:c r="C106" s="143" t="str">
         <x:f>IF(A106="","",'課題入力'!E106)</x:f>
       </x:c>
     </x:row>
-    <x:row r="107">
-      <x:c r="A107" s="112" t="str">
+    <x:row r="107" ht="24" customHeight="1">
+      <x:c r="A107" s="141" t="str">
         <x:f>IF('課題入力'!H107=1,'課題入力'!A107,"")</x:f>
       </x:c>
-      <x:c r="B107" s="113" t="str">
+      <x:c r="B107" s="142" t="str">
         <x:f>IF(A107="","",'課題入力'!B107)</x:f>
       </x:c>
-      <x:c r="C107" s="114" t="str">
+      <x:c r="C107" s="143" t="str">
         <x:f>IF(A107="","",'課題入力'!E107)</x:f>
       </x:c>
     </x:row>
-    <x:row r="108">
-      <x:c r="A108" s="112" t="str">
+    <x:row r="108" ht="24" customHeight="1">
+      <x:c r="A108" s="141" t="str">
         <x:f>IF('課題入力'!H108=1,'課題入力'!A108,"")</x:f>
       </x:c>
-      <x:c r="B108" s="113" t="str">
+      <x:c r="B108" s="142" t="str">
         <x:f>IF(A108="","",'課題入力'!B108)</x:f>
       </x:c>
-      <x:c r="C108" s="114" t="str">
+      <x:c r="C108" s="143" t="str">
         <x:f>IF(A108="","",'課題入力'!E108)</x:f>
       </x:c>
     </x:row>
-    <x:row r="109">
-      <x:c r="A109" s="112" t="str">
+    <x:row r="109" ht="24" customHeight="1">
+      <x:c r="A109" s="141" t="str">
         <x:f>IF('課題入力'!H109=1,'課題入力'!A109,"")</x:f>
       </x:c>
-      <x:c r="B109" s="113" t="str">
+      <x:c r="B109" s="142" t="str">
         <x:f>IF(A109="","",'課題入力'!B109)</x:f>
       </x:c>
-      <x:c r="C109" s="114" t="str">
+      <x:c r="C109" s="143" t="str">
         <x:f>IF(A109="","",'課題入力'!E109)</x:f>
       </x:c>
     </x:row>
-    <x:row r="110">
-      <x:c r="A110" s="112" t="str">
+    <x:row r="110" ht="24" customHeight="1">
+      <x:c r="A110" s="141" t="str">
         <x:f>IF('課題入力'!H110=1,'課題入力'!A110,"")</x:f>
       </x:c>
-      <x:c r="B110" s="113" t="str">
+      <x:c r="B110" s="142" t="str">
         <x:f>IF(A110="","",'課題入力'!B110)</x:f>
       </x:c>
-      <x:c r="C110" s="114" t="str">
+      <x:c r="C110" s="143" t="str">
         <x:f>IF(A110="","",'課題入力'!E110)</x:f>
       </x:c>
     </x:row>
-    <x:row r="111">
-      <x:c r="A111" s="112" t="str">
+    <x:row r="111" ht="24" customHeight="1">
+      <x:c r="A111" s="141" t="str">
         <x:f>IF('課題入力'!H111=1,'課題入力'!A111,"")</x:f>
       </x:c>
-      <x:c r="B111" s="113" t="str">
+      <x:c r="B111" s="142" t="str">
         <x:f>IF(A111="","",'課題入力'!B111)</x:f>
       </x:c>
-      <x:c r="C111" s="114" t="str">
+      <x:c r="C111" s="143" t="str">
         <x:f>IF(A111="","",'課題入力'!E111)</x:f>
       </x:c>
     </x:row>
-    <x:row r="112">
-      <x:c r="A112" s="112" t="str">
+    <x:row r="112" ht="24" customHeight="1">
+      <x:c r="A112" s="141" t="str">
         <x:f>IF('課題入力'!H112=1,'課題入力'!A112,"")</x:f>
       </x:c>
-      <x:c r="B112" s="113" t="str">
+      <x:c r="B112" s="142" t="str">
         <x:f>IF(A112="","",'課題入力'!B112)</x:f>
       </x:c>
-      <x:c r="C112" s="114" t="str">
+      <x:c r="C112" s="143" t="str">
         <x:f>IF(A112="","",'課題入力'!E112)</x:f>
       </x:c>
     </x:row>
-    <x:row r="113">
-      <x:c r="A113" s="112" t="str">
+    <x:row r="113" ht="24" customHeight="1">
+      <x:c r="A113" s="141" t="str">
         <x:f>IF('課題入力'!H113=1,'課題入力'!A113,"")</x:f>
       </x:c>
-      <x:c r="B113" s="113" t="str">
+      <x:c r="B113" s="142" t="str">
         <x:f>IF(A113="","",'課題入力'!B113)</x:f>
       </x:c>
-      <x:c r="C113" s="114" t="str">
+      <x:c r="C113" s="143" t="str">
         <x:f>IF(A113="","",'課題入力'!E113)</x:f>
       </x:c>
     </x:row>
-    <x:row r="114">
-      <x:c r="A114" s="112" t="str">
+    <x:row r="114" ht="24" customHeight="1">
+      <x:c r="A114" s="141" t="str">
         <x:f>IF('課題入力'!H114=1,'課題入力'!A114,"")</x:f>
       </x:c>
-      <x:c r="B114" s="113" t="str">
+      <x:c r="B114" s="142" t="str">
         <x:f>IF(A114="","",'課題入力'!B114)</x:f>
       </x:c>
-      <x:c r="C114" s="114" t="str">
+      <x:c r="C114" s="143" t="str">
         <x:f>IF(A114="","",'課題入力'!E114)</x:f>
       </x:c>
     </x:row>
-    <x:row r="115">
-      <x:c r="A115" s="112" t="str">
+    <x:row r="115" ht="24" customHeight="1">
+      <x:c r="A115" s="141" t="str">
         <x:f>IF('課題入力'!H115=1,'課題入力'!A115,"")</x:f>
       </x:c>
-      <x:c r="B115" s="113" t="str">
+      <x:c r="B115" s="142" t="str">
         <x:f>IF(A115="","",'課題入力'!B115)</x:f>
       </x:c>
-      <x:c r="C115" s="114" t="str">
+      <x:c r="C115" s="143" t="str">
         <x:f>IF(A115="","",'課題入力'!E115)</x:f>
       </x:c>
     </x:row>
-    <x:row r="116">
-      <x:c r="A116" s="112" t="str">
+    <x:row r="116" ht="24" customHeight="1">
+      <x:c r="A116" s="141" t="str">
         <x:f>IF('課題入力'!H116=1,'課題入力'!A116,"")</x:f>
       </x:c>
-      <x:c r="B116" s="113" t="str">
+      <x:c r="B116" s="142" t="str">
         <x:f>IF(A116="","",'課題入力'!B116)</x:f>
       </x:c>
-      <x:c r="C116" s="114" t="str">
+      <x:c r="C116" s="143" t="str">
         <x:f>IF(A116="","",'課題入力'!E116)</x:f>
       </x:c>
     </x:row>
-    <x:row r="117">
-      <x:c r="A117" s="112" t="str">
+    <x:row r="117" ht="24" customHeight="1">
+      <x:c r="A117" s="141" t="str">
         <x:f>IF('課題入力'!H117=1,'課題入力'!A117,"")</x:f>
       </x:c>
-      <x:c r="B117" s="113" t="str">
+      <x:c r="B117" s="142" t="str">
         <x:f>IF(A117="","",'課題入力'!B117)</x:f>
       </x:c>
-      <x:c r="C117" s="114" t="str">
+      <x:c r="C117" s="143" t="str">
         <x:f>IF(A117="","",'課題入力'!E117)</x:f>
       </x:c>
     </x:row>
-    <x:row r="118">
-      <x:c r="A118" s="112" t="str">
+    <x:row r="118" ht="24" customHeight="1">
+      <x:c r="A118" s="141" t="str">
         <x:f>IF('課題入力'!H118=1,'課題入力'!A118,"")</x:f>
       </x:c>
-      <x:c r="B118" s="113" t="str">
+      <x:c r="B118" s="142" t="str">
         <x:f>IF(A118="","",'課題入力'!B118)</x:f>
       </x:c>
-      <x:c r="C118" s="114" t="str">
+      <x:c r="C118" s="143" t="str">
         <x:f>IF(A118="","",'課題入力'!E118)</x:f>
       </x:c>
     </x:row>
-    <x:row r="119">
-      <x:c r="A119" s="112" t="str">
+    <x:row r="119" ht="24" customHeight="1">
+      <x:c r="A119" s="141" t="str">
         <x:f>IF('課題入力'!H119=1,'課題入力'!A119,"")</x:f>
       </x:c>
-      <x:c r="B119" s="113" t="str">
+      <x:c r="B119" s="142" t="str">
         <x:f>IF(A119="","",'課題入力'!B119)</x:f>
       </x:c>
-      <x:c r="C119" s="114" t="str">
+      <x:c r="C119" s="143" t="str">
         <x:f>IF(A119="","",'課題入力'!E119)</x:f>
       </x:c>
     </x:row>
-    <x:row r="120">
-      <x:c r="A120" s="112" t="str">
+    <x:row r="120" ht="24" customHeight="1">
+      <x:c r="A120" s="141" t="str">
         <x:f>IF('課題入力'!H120=1,'課題入力'!A120,"")</x:f>
       </x:c>
-      <x:c r="B120" s="113" t="str">
+      <x:c r="B120" s="142" t="str">
         <x:f>IF(A120="","",'課題入力'!B120)</x:f>
       </x:c>
-      <x:c r="C120" s="114" t="str">
+      <x:c r="C120" s="143" t="str">
         <x:f>IF(A120="","",'課題入力'!E120)</x:f>
       </x:c>
     </x:row>
-    <x:row r="121">
-      <x:c r="A121" s="112" t="str">
+    <x:row r="121" ht="24" customHeight="1">
+      <x:c r="A121" s="141" t="str">
         <x:f>IF('課題入力'!H121=1,'課題入力'!A121,"")</x:f>
       </x:c>
-      <x:c r="B121" s="113" t="str">
+      <x:c r="B121" s="142" t="str">
         <x:f>IF(A121="","",'課題入力'!B121)</x:f>
       </x:c>
-      <x:c r="C121" s="114" t="str">
+      <x:c r="C121" s="143" t="str">
         <x:f>IF(A121="","",'課題入力'!E121)</x:f>
       </x:c>
     </x:row>
-    <x:row r="122">
-      <x:c r="A122" s="112" t="str">
+    <x:row r="122" ht="24" customHeight="1">
+      <x:c r="A122" s="141" t="str">
         <x:f>IF('課題入力'!H122=1,'課題入力'!A122,"")</x:f>
       </x:c>
-      <x:c r="B122" s="113" t="str">
+      <x:c r="B122" s="142" t="str">
         <x:f>IF(A122="","",'課題入力'!B122)</x:f>
       </x:c>
-      <x:c r="C122" s="114" t="str">
+      <x:c r="C122" s="143" t="str">
         <x:f>IF(A122="","",'課題入力'!E122)</x:f>
       </x:c>
     </x:row>
-    <x:row r="123">
-      <x:c r="A123" s="112" t="str">
+    <x:row r="123" ht="24" customHeight="1">
+      <x:c r="A123" s="141" t="str">
         <x:f>IF('課題入力'!H123=1,'課題入力'!A123,"")</x:f>
       </x:c>
-      <x:c r="B123" s="113" t="str">
+      <x:c r="B123" s="142" t="str">
         <x:f>IF(A123="","",'課題入力'!B123)</x:f>
       </x:c>
-      <x:c r="C123" s="114" t="str">
+      <x:c r="C123" s="143" t="str">
         <x:f>IF(A123="","",'課題入力'!E123)</x:f>
       </x:c>
     </x:row>
-    <x:row r="124">
-      <x:c r="A124" s="112" t="str">
+    <x:row r="124" ht="24" customHeight="1">
+      <x:c r="A124" s="141" t="str">
         <x:f>IF('課題入力'!H124=1,'課題入力'!A124,"")</x:f>
       </x:c>
-      <x:c r="B124" s="113" t="str">
+      <x:c r="B124" s="142" t="str">
         <x:f>IF(A124="","",'課題入力'!B124)</x:f>
       </x:c>
-      <x:c r="C124" s="114" t="str">
+      <x:c r="C124" s="143" t="str">
         <x:f>IF(A124="","",'課題入力'!E124)</x:f>
       </x:c>
     </x:row>
-    <x:row r="125">
-      <x:c r="A125" s="112" t="str">
+    <x:row r="125" ht="24" customHeight="1">
+      <x:c r="A125" s="141" t="str">
         <x:f>IF('課題入力'!H125=1,'課題入力'!A125,"")</x:f>
       </x:c>
-      <x:c r="B125" s="113" t="str">
+      <x:c r="B125" s="142" t="str">
         <x:f>IF(A125="","",'課題入力'!B125)</x:f>
       </x:c>
-      <x:c r="C125" s="114" t="str">
+      <x:c r="C125" s="143" t="str">
         <x:f>IF(A125="","",'課題入力'!E125)</x:f>
       </x:c>
     </x:row>
-    <x:row r="126">
-      <x:c r="A126" s="112" t="str">
+    <x:row r="126" ht="24" customHeight="1">
+      <x:c r="A126" s="141" t="str">
         <x:f>IF('課題入力'!H126=1,'課題入力'!A126,"")</x:f>
       </x:c>
-      <x:c r="B126" s="113" t="str">
+      <x:c r="B126" s="142" t="str">
         <x:f>IF(A126="","",'課題入力'!B126)</x:f>
       </x:c>
-      <x:c r="C126" s="114" t="str">
+      <x:c r="C126" s="143" t="str">
         <x:f>IF(A126="","",'課題入力'!E126)</x:f>
       </x:c>
     </x:row>
-    <x:row r="127">
-      <x:c r="A127" s="112" t="str">
+    <x:row r="127" ht="24" customHeight="1">
+      <x:c r="A127" s="141" t="str">
         <x:f>IF('課題入力'!H127=1,'課題入力'!A127,"")</x:f>
       </x:c>
-      <x:c r="B127" s="113" t="str">
+      <x:c r="B127" s="142" t="str">
         <x:f>IF(A127="","",'課題入力'!B127)</x:f>
       </x:c>
-      <x:c r="C127" s="114" t="str">
+      <x:c r="C127" s="143" t="str">
         <x:f>IF(A127="","",'課題入力'!E127)</x:f>
       </x:c>
     </x:row>
-    <x:row r="128">
-      <x:c r="A128" s="112" t="str">
+    <x:row r="128" ht="24" customHeight="1">
+      <x:c r="A128" s="141" t="str">
         <x:f>IF('課題入力'!H128=1,'課題入力'!A128,"")</x:f>
       </x:c>
-      <x:c r="B128" s="113" t="str">
+      <x:c r="B128" s="142" t="str">
         <x:f>IF(A128="","",'課題入力'!B128)</x:f>
       </x:c>
-      <x:c r="C128" s="114" t="str">
+      <x:c r="C128" s="143" t="str">
         <x:f>IF(A128="","",'課題入力'!E128)</x:f>
       </x:c>
     </x:row>
-    <x:row r="129">
-      <x:c r="A129" s="112" t="str">
+    <x:row r="129" ht="24" customHeight="1">
+      <x:c r="A129" s="141" t="str">
         <x:f>IF('課題入力'!H129=1,'課題入力'!A129,"")</x:f>
       </x:c>
-      <x:c r="B129" s="113" t="str">
+      <x:c r="B129" s="142" t="str">
         <x:f>IF(A129="","",'課題入力'!B129)</x:f>
       </x:c>
-      <x:c r="C129" s="114" t="str">
+      <x:c r="C129" s="143" t="str">
         <x:f>IF(A129="","",'課題入力'!E129)</x:f>
       </x:c>
     </x:row>
-    <x:row r="130">
-      <x:c r="A130" s="112" t="str">
+    <x:row r="130" ht="24" customHeight="1">
+      <x:c r="A130" s="141" t="str">
         <x:f>IF('課題入力'!H130=1,'課題入力'!A130,"")</x:f>
       </x:c>
-      <x:c r="B130" s="113" t="str">
+      <x:c r="B130" s="142" t="str">
         <x:f>IF(A130="","",'課題入力'!B130)</x:f>
       </x:c>
-      <x:c r="C130" s="114" t="str">
+      <x:c r="C130" s="143" t="str">
         <x:f>IF(A130="","",'課題入力'!E130)</x:f>
       </x:c>
     </x:row>
-    <x:row r="131">
-      <x:c r="A131" s="112" t="str">
+    <x:row r="131" ht="24" customHeight="1">
+      <x:c r="A131" s="141" t="str">
         <x:f>IF('課題入力'!H131=1,'課題入力'!A131,"")</x:f>
       </x:c>
-      <x:c r="B131" s="113" t="str">
+      <x:c r="B131" s="142" t="str">
         <x:f>IF(A131="","",'課題入力'!B131)</x:f>
       </x:c>
-      <x:c r="C131" s="114" t="str">
+      <x:c r="C131" s="143" t="str">
         <x:f>IF(A131="","",'課題入力'!E131)</x:f>
       </x:c>
     </x:row>
-    <x:row r="132">
-      <x:c r="A132" s="112" t="str">
+    <x:row r="132" ht="24" customHeight="1">
+      <x:c r="A132" s="141" t="str">
         <x:f>IF('課題入力'!H132=1,'課題入力'!A132,"")</x:f>
       </x:c>
-      <x:c r="B132" s="113" t="str">
+      <x:c r="B132" s="142" t="str">
         <x:f>IF(A132="","",'課題入力'!B132)</x:f>
       </x:c>
-      <x:c r="C132" s="114" t="str">
+      <x:c r="C132" s="143" t="str">
         <x:f>IF(A132="","",'課題入力'!E132)</x:f>
       </x:c>
     </x:row>
-    <x:row r="133">
-      <x:c r="A133" s="112" t="str">
+    <x:row r="133" ht="24" customHeight="1">
+      <x:c r="A133" s="141" t="str">
         <x:f>IF('課題入力'!H133=1,'課題入力'!A133,"")</x:f>
       </x:c>
-      <x:c r="B133" s="113" t="str">
+      <x:c r="B133" s="142" t="str">
         <x:f>IF(A133="","",'課題入力'!B133)</x:f>
       </x:c>
-      <x:c r="C133" s="114" t="str">
+      <x:c r="C133" s="143" t="str">
         <x:f>IF(A133="","",'課題入力'!E133)</x:f>
       </x:c>
     </x:row>
-    <x:row r="134">
-      <x:c r="A134" s="112" t="str">
+    <x:row r="134" ht="24" customHeight="1">
+      <x:c r="A134" s="141" t="str">
         <x:f>IF('課題入力'!H134=1,'課題入力'!A134,"")</x:f>
       </x:c>
-      <x:c r="B134" s="113" t="str">
+      <x:c r="B134" s="142" t="str">
         <x:f>IF(A134="","",'課題入力'!B134)</x:f>
       </x:c>
-      <x:c r="C134" s="114" t="str">
+      <x:c r="C134" s="143" t="str">
         <x:f>IF(A134="","",'課題入力'!E134)</x:f>
       </x:c>
     </x:row>
-    <x:row r="135">
-      <x:c r="A135" s="112" t="str">
+    <x:row r="135" ht="24" customHeight="1">
+      <x:c r="A135" s="141" t="str">
         <x:f>IF('課題入力'!H135=1,'課題入力'!A135,"")</x:f>
       </x:c>
-      <x:c r="B135" s="113" t="str">
+      <x:c r="B135" s="142" t="str">
         <x:f>IF(A135="","",'課題入力'!B135)</x:f>
       </x:c>
-      <x:c r="C135" s="114" t="str">
+      <x:c r="C135" s="143" t="str">
         <x:f>IF(A135="","",'課題入力'!E135)</x:f>
       </x:c>
     </x:row>
-    <x:row r="136">
-      <x:c r="A136" s="112" t="str">
+    <x:row r="136" ht="24" customHeight="1">
+      <x:c r="A136" s="141" t="str">
         <x:f>IF('課題入力'!H136=1,'課題入力'!A136,"")</x:f>
       </x:c>
-      <x:c r="B136" s="113" t="str">
+      <x:c r="B136" s="142" t="str">
         <x:f>IF(A136="","",'課題入力'!B136)</x:f>
       </x:c>
-      <x:c r="C136" s="114" t="str">
+      <x:c r="C136" s="143" t="str">
         <x:f>IF(A136="","",'課題入力'!E136)</x:f>
       </x:c>
     </x:row>
-    <x:row r="137">
-      <x:c r="A137" s="112" t="str">
+    <x:row r="137" ht="24" customHeight="1">
+      <x:c r="A137" s="141" t="str">
         <x:f>IF('課題入力'!H137=1,'課題入力'!A137,"")</x:f>
       </x:c>
-      <x:c r="B137" s="113" t="str">
+      <x:c r="B137" s="142" t="str">
         <x:f>IF(A137="","",'課題入力'!B137)</x:f>
       </x:c>
-      <x:c r="C137" s="114" t="str">
+      <x:c r="C137" s="143" t="str">
         <x:f>IF(A137="","",'課題入力'!E137)</x:f>
       </x:c>
     </x:row>
-    <x:row r="138">
-      <x:c r="A138" s="112" t="str">
+    <x:row r="138" ht="24" customHeight="1">
+      <x:c r="A138" s="141" t="str">
         <x:f>IF('課題入力'!H138=1,'課題入力'!A138,"")</x:f>
       </x:c>
-      <x:c r="B138" s="113" t="str">
+      <x:c r="B138" s="142" t="str">
         <x:f>IF(A138="","",'課題入力'!B138)</x:f>
       </x:c>
-      <x:c r="C138" s="114" t="str">
+      <x:c r="C138" s="143" t="str">
         <x:f>IF(A138="","",'課題入力'!E138)</x:f>
       </x:c>
     </x:row>
-    <x:row r="139">
-      <x:c r="A139" s="112" t="str">
+    <x:row r="139" ht="24" customHeight="1">
+      <x:c r="A139" s="141" t="str">
         <x:f>IF('課題入力'!H139=1,'課題入力'!A139,"")</x:f>
       </x:c>
-      <x:c r="B139" s="113" t="str">
+      <x:c r="B139" s="142" t="str">
         <x:f>IF(A139="","",'課題入力'!B139)</x:f>
       </x:c>
-      <x:c r="C139" s="114" t="str">
+      <x:c r="C139" s="143" t="str">
         <x:f>IF(A139="","",'課題入力'!E139)</x:f>
       </x:c>
     </x:row>
-    <x:row r="140">
-      <x:c r="A140" s="112" t="str">
+    <x:row r="140" ht="24" customHeight="1">
+      <x:c r="A140" s="141" t="str">
         <x:f>IF('課題入力'!H140=1,'課題入力'!A140,"")</x:f>
       </x:c>
-      <x:c r="B140" s="113" t="str">
+      <x:c r="B140" s="142" t="str">
         <x:f>IF(A140="","",'課題入力'!B140)</x:f>
       </x:c>
-      <x:c r="C140" s="114" t="str">
+      <x:c r="C140" s="143" t="str">
         <x:f>IF(A140="","",'課題入力'!E140)</x:f>
       </x:c>
     </x:row>
-    <x:row r="141">
-      <x:c r="A141" s="112" t="str">
+    <x:row r="141" ht="24" customHeight="1">
+      <x:c r="A141" s="141" t="str">
         <x:f>IF('課題入力'!H141=1,'課題入力'!A141,"")</x:f>
       </x:c>
-      <x:c r="B141" s="113" t="str">
+      <x:c r="B141" s="142" t="str">
         <x:f>IF(A141="","",'課題入力'!B141)</x:f>
       </x:c>
-      <x:c r="C141" s="114" t="str">
+      <x:c r="C141" s="143" t="str">
         <x:f>IF(A141="","",'課題入力'!E141)</x:f>
       </x:c>
     </x:row>
-    <x:row r="142">
-      <x:c r="A142" s="112" t="str">
+    <x:row r="142" ht="24" customHeight="1">
+      <x:c r="A142" s="141" t="str">
         <x:f>IF('課題入力'!H142=1,'課題入力'!A142,"")</x:f>
       </x:c>
-      <x:c r="B142" s="113" t="str">
+      <x:c r="B142" s="142" t="str">
         <x:f>IF(A142="","",'課題入力'!B142)</x:f>
       </x:c>
-      <x:c r="C142" s="114" t="str">
+      <x:c r="C142" s="143" t="str">
         <x:f>IF(A142="","",'課題入力'!E142)</x:f>
       </x:c>
     </x:row>
-    <x:row r="143">
-      <x:c r="A143" s="112" t="str">
+    <x:row r="143" ht="24" customHeight="1">
+      <x:c r="A143" s="141" t="str">
         <x:f>IF('課題入力'!H143=1,'課題入力'!A143,"")</x:f>
       </x:c>
-      <x:c r="B143" s="113" t="str">
+      <x:c r="B143" s="142" t="str">
         <x:f>IF(A143="","",'課題入力'!B143)</x:f>
       </x:c>
-      <x:c r="C143" s="114" t="str">
+      <x:c r="C143" s="143" t="str">
         <x:f>IF(A143="","",'課題入力'!E143)</x:f>
       </x:c>
     </x:row>
-    <x:row r="144">
-      <x:c r="A144" s="112" t="str">
+    <x:row r="144" ht="24" customHeight="1">
+      <x:c r="A144" s="141" t="str">
         <x:f>IF('課題入力'!H144=1,'課題入力'!A144,"")</x:f>
       </x:c>
-      <x:c r="B144" s="113" t="str">
+      <x:c r="B144" s="142" t="str">
         <x:f>IF(A144="","",'課題入力'!B144)</x:f>
       </x:c>
-      <x:c r="C144" s="114" t="str">
+      <x:c r="C144" s="143" t="str">
         <x:f>IF(A144="","",'課題入力'!E144)</x:f>
       </x:c>
     </x:row>
-    <x:row r="145">
-      <x:c r="A145" s="112" t="str">
+    <x:row r="145" ht="24" customHeight="1">
+      <x:c r="A145" s="141" t="str">
         <x:f>IF('課題入力'!H145=1,'課題入力'!A145,"")</x:f>
       </x:c>
-      <x:c r="B145" s="113" t="str">
+      <x:c r="B145" s="142" t="str">
         <x:f>IF(A145="","",'課題入力'!B145)</x:f>
       </x:c>
-      <x:c r="C145" s="114" t="str">
+      <x:c r="C145" s="143" t="str">
         <x:f>IF(A145="","",'課題入力'!E145)</x:f>
       </x:c>
     </x:row>
-    <x:row r="146">
-      <x:c r="A146" s="112" t="str">
+    <x:row r="146" ht="24" customHeight="1">
+      <x:c r="A146" s="141" t="str">
         <x:f>IF('課題入力'!H146=1,'課題入力'!A146,"")</x:f>
       </x:c>
-      <x:c r="B146" s="113" t="str">
+      <x:c r="B146" s="142" t="str">
         <x:f>IF(A146="","",'課題入力'!B146)</x:f>
       </x:c>
-      <x:c r="C146" s="114" t="str">
+      <x:c r="C146" s="143" t="str">
         <x:f>IF(A146="","",'課題入力'!E146)</x:f>
       </x:c>
     </x:row>
-    <x:row r="147">
-      <x:c r="A147" s="112" t="str">
+    <x:row r="147" ht="24" customHeight="1">
+      <x:c r="A147" s="141" t="str">
         <x:f>IF('課題入力'!H147=1,'課題入力'!A147,"")</x:f>
       </x:c>
-      <x:c r="B147" s="113" t="str">
+      <x:c r="B147" s="142" t="str">
         <x:f>IF(A147="","",'課題入力'!B147)</x:f>
       </x:c>
-      <x:c r="C147" s="114" t="str">
+      <x:c r="C147" s="143" t="str">
         <x:f>IF(A147="","",'課題入力'!E147)</x:f>
       </x:c>
     </x:row>
-    <x:row r="148">
-      <x:c r="A148" s="112" t="str">
+    <x:row r="148" ht="24" customHeight="1">
+      <x:c r="A148" s="141" t="str">
         <x:f>IF('課題入力'!H148=1,'課題入力'!A148,"")</x:f>
       </x:c>
-      <x:c r="B148" s="113" t="str">
+      <x:c r="B148" s="142" t="str">
         <x:f>IF(A148="","",'課題入力'!B148)</x:f>
       </x:c>
-      <x:c r="C148" s="114" t="str">
+      <x:c r="C148" s="143" t="str">
         <x:f>IF(A148="","",'課題入力'!E148)</x:f>
       </x:c>
     </x:row>
-    <x:row r="149">
-      <x:c r="A149" s="112" t="str">
+    <x:row r="149" ht="24" customHeight="1">
+      <x:c r="A149" s="141" t="str">
         <x:f>IF('課題入力'!H149=1,'課題入力'!A149,"")</x:f>
       </x:c>
-      <x:c r="B149" s="113" t="str">
+      <x:c r="B149" s="142" t="str">
         <x:f>IF(A149="","",'課題入力'!B149)</x:f>
       </x:c>
-      <x:c r="C149" s="114" t="str">
+      <x:c r="C149" s="143" t="str">
         <x:f>IF(A149="","",'課題入力'!E149)</x:f>
       </x:c>
     </x:row>
-    <x:row r="150">
-      <x:c r="A150" s="112" t="str">
+    <x:row r="150" ht="24" customHeight="1">
+      <x:c r="A150" s="141" t="str">
         <x:f>IF('課題入力'!H150=1,'課題入力'!A150,"")</x:f>
       </x:c>
-      <x:c r="B150" s="113" t="str">
+      <x:c r="B150" s="142" t="str">
         <x:f>IF(A150="","",'課題入力'!B150)</x:f>
       </x:c>
-      <x:c r="C150" s="114" t="str">
+      <x:c r="C150" s="143" t="str">
         <x:f>IF(A150="","",'課題入力'!E150)</x:f>
       </x:c>
     </x:row>
-    <x:row r="151">
-      <x:c r="A151" s="112" t="str">
+    <x:row r="151" ht="24" customHeight="1">
+      <x:c r="A151" s="141" t="str">
         <x:f>IF('課題入力'!H151=1,'課題入力'!A151,"")</x:f>
       </x:c>
-      <x:c r="B151" s="113" t="str">
+      <x:c r="B151" s="142" t="str">
         <x:f>IF(A151="","",'課題入力'!B151)</x:f>
       </x:c>
-      <x:c r="C151" s="114" t="str">
+      <x:c r="C151" s="143" t="str">
         <x:f>IF(A151="","",'課題入力'!E151)</x:f>
       </x:c>
     </x:row>
-    <x:row r="152">
-      <x:c r="A152" s="112" t="str">
+    <x:row r="152" ht="24" customHeight="1">
+      <x:c r="A152" s="141" t="str">
         <x:f>IF('課題入力'!H152=1,'課題入力'!A152,"")</x:f>
       </x:c>
-      <x:c r="B152" s="113" t="str">
+      <x:c r="B152" s="142" t="str">
         <x:f>IF(A152="","",'課題入力'!B152)</x:f>
       </x:c>
-      <x:c r="C152" s="114" t="str">
+      <x:c r="C152" s="143" t="str">
         <x:f>IF(A152="","",'課題入力'!E152)</x:f>
       </x:c>
     </x:row>
-    <x:row r="153">
-      <x:c r="A153" s="112" t="str">
+    <x:row r="153" ht="24" customHeight="1">
+      <x:c r="A153" s="141" t="str">
         <x:f>IF('課題入力'!H153=1,'課題入力'!A153,"")</x:f>
       </x:c>
-      <x:c r="B153" s="113" t="str">
+      <x:c r="B153" s="142" t="str">
         <x:f>IF(A153="","",'課題入力'!B153)</x:f>
       </x:c>
-      <x:c r="C153" s="114" t="str">
+      <x:c r="C153" s="143" t="str">
         <x:f>IF(A153="","",'課題入力'!E153)</x:f>
       </x:c>
     </x:row>
-    <x:row r="154">
-      <x:c r="A154" s="112" t="str">
+    <x:row r="154" ht="24" customHeight="1">
+      <x:c r="A154" s="141" t="str">
         <x:f>IF('課題入力'!H154=1,'課題入力'!A154,"")</x:f>
       </x:c>
-      <x:c r="B154" s="113" t="str">
+      <x:c r="B154" s="142" t="str">
         <x:f>IF(A154="","",'課題入力'!B154)</x:f>
       </x:c>
-      <x:c r="C154" s="114" t="str">
+      <x:c r="C154" s="143" t="str">
         <x:f>IF(A154="","",'課題入力'!E154)</x:f>
       </x:c>
     </x:row>
-    <x:row r="155">
-      <x:c r="A155" s="112" t="str">
+    <x:row r="155" ht="24" customHeight="1">
+      <x:c r="A155" s="141" t="str">
         <x:f>IF('課題入力'!H155=1,'課題入力'!A155,"")</x:f>
       </x:c>
-      <x:c r="B155" s="113" t="str">
+      <x:c r="B155" s="142" t="str">
         <x:f>IF(A155="","",'課題入力'!B155)</x:f>
       </x:c>
-      <x:c r="C155" s="114" t="str">
+      <x:c r="C155" s="143" t="str">
         <x:f>IF(A155="","",'課題入力'!E155)</x:f>
       </x:c>
     </x:row>
-    <x:row r="156">
-      <x:c r="A156" s="112" t="str">
+    <x:row r="156" ht="24" customHeight="1">
+      <x:c r="A156" s="141" t="str">
         <x:f>IF('課題入力'!H156=1,'課題入力'!A156,"")</x:f>
       </x:c>
-      <x:c r="B156" s="113" t="str">
+      <x:c r="B156" s="142" t="str">
         <x:f>IF(A156="","",'課題入力'!B156)</x:f>
       </x:c>
-      <x:c r="C156" s="114" t="str">
+      <x:c r="C156" s="143" t="str">
         <x:f>IF(A156="","",'課題入力'!E156)</x:f>
       </x:c>
     </x:row>
-    <x:row r="157">
-      <x:c r="A157" s="112" t="str">
+    <x:row r="157" ht="24" customHeight="1">
+      <x:c r="A157" s="141" t="str">
         <x:f>IF('課題入力'!H157=1,'課題入力'!A157,"")</x:f>
       </x:c>
-      <x:c r="B157" s="113" t="str">
+      <x:c r="B157" s="142" t="str">
         <x:f>IF(A157="","",'課題入力'!B157)</x:f>
       </x:c>
-      <x:c r="C157" s="114" t="str">
+      <x:c r="C157" s="143" t="str">
         <x:f>IF(A157="","",'課題入力'!E157)</x:f>
       </x:c>
     </x:row>
-    <x:row r="158">
-      <x:c r="A158" s="112" t="str">
+    <x:row r="158" ht="24" customHeight="1">
+      <x:c r="A158" s="141" t="str">
         <x:f>IF('課題入力'!H158=1,'課題入力'!A158,"")</x:f>
       </x:c>
-      <x:c r="B158" s="113" t="str">
+      <x:c r="B158" s="142" t="str">
         <x:f>IF(A158="","",'課題入力'!B158)</x:f>
       </x:c>
-      <x:c r="C158" s="114" t="str">
+      <x:c r="C158" s="143" t="str">
         <x:f>IF(A158="","",'課題入力'!E158)</x:f>
       </x:c>
     </x:row>
-    <x:row r="159">
-      <x:c r="A159" s="112" t="str">
+    <x:row r="159" ht="24" customHeight="1">
+      <x:c r="A159" s="141" t="str">
         <x:f>IF('課題入力'!H159=1,'課題入力'!A159,"")</x:f>
       </x:c>
-      <x:c r="B159" s="113" t="str">
+      <x:c r="B159" s="142" t="str">
         <x:f>IF(A159="","",'課題入力'!B159)</x:f>
       </x:c>
-      <x:c r="C159" s="114" t="str">
+      <x:c r="C159" s="143" t="str">
         <x:f>IF(A159="","",'課題入力'!E159)</x:f>
       </x:c>
     </x:row>
-    <x:row r="160">
-      <x:c r="A160" s="112" t="str">
+    <x:row r="160" ht="24" customHeight="1">
+      <x:c r="A160" s="141" t="str">
         <x:f>IF('課題入力'!H160=1,'課題入力'!A160,"")</x:f>
       </x:c>
-      <x:c r="B160" s="113" t="str">
+      <x:c r="B160" s="142" t="str">
         <x:f>IF(A160="","",'課題入力'!B160)</x:f>
       </x:c>
-      <x:c r="C160" s="114" t="str">
+      <x:c r="C160" s="143" t="str">
         <x:f>IF(A160="","",'課題入力'!E160)</x:f>
       </x:c>
     </x:row>
-    <x:row r="161">
-      <x:c r="A161" s="112" t="str">
+    <x:row r="161" ht="24" customHeight="1">
+      <x:c r="A161" s="141" t="str">
         <x:f>IF('課題入力'!H161=1,'課題入力'!A161,"")</x:f>
       </x:c>
-      <x:c r="B161" s="113" t="str">
+      <x:c r="B161" s="142" t="str">
         <x:f>IF(A161="","",'課題入力'!B161)</x:f>
       </x:c>
-      <x:c r="C161" s="114" t="str">
+      <x:c r="C161" s="143" t="str">
         <x:f>IF(A161="","",'課題入力'!E161)</x:f>
       </x:c>
     </x:row>
-    <x:row r="162">
-      <x:c r="A162" s="112" t="str">
+    <x:row r="162" ht="24" customHeight="1">
+      <x:c r="A162" s="141" t="str">
         <x:f>IF('課題入力'!H162=1,'課題入力'!A162,"")</x:f>
       </x:c>
-      <x:c r="B162" s="113" t="str">
+      <x:c r="B162" s="142" t="str">
         <x:f>IF(A162="","",'課題入力'!B162)</x:f>
       </x:c>
-      <x:c r="C162" s="114" t="str">
+      <x:c r="C162" s="143" t="str">
         <x:f>IF(A162="","",'課題入力'!E162)</x:f>
       </x:c>
     </x:row>
-    <x:row r="163">
-      <x:c r="A163" s="112" t="str">
+    <x:row r="163" ht="24" customHeight="1">
+      <x:c r="A163" s="141" t="str">
         <x:f>IF('課題入力'!H163=1,'課題入力'!A163,"")</x:f>
       </x:c>
-      <x:c r="B163" s="113" t="str">
+      <x:c r="B163" s="142" t="str">
         <x:f>IF(A163="","",'課題入力'!B163)</x:f>
       </x:c>
-      <x:c r="C163" s="114" t="str">
+      <x:c r="C163" s="143" t="str">
         <x:f>IF(A163="","",'課題入力'!E163)</x:f>
       </x:c>
     </x:row>
-    <x:row r="164">
-      <x:c r="A164" s="112" t="str">
+    <x:row r="164" ht="24" customHeight="1">
+      <x:c r="A164" s="141" t="str">
         <x:f>IF('課題入力'!H164=1,'課題入力'!A164,"")</x:f>
       </x:c>
-      <x:c r="B164" s="113" t="str">
+      <x:c r="B164" s="142" t="str">
         <x:f>IF(A164="","",'課題入力'!B164)</x:f>
       </x:c>
-      <x:c r="C164" s="114" t="str">
+      <x:c r="C164" s="143" t="str">
         <x:f>IF(A164="","",'課題入力'!E164)</x:f>
       </x:c>
     </x:row>
-    <x:row r="165">
-      <x:c r="A165" s="112" t="str">
+    <x:row r="165" ht="24" customHeight="1">
+      <x:c r="A165" s="141" t="str">
         <x:f>IF('課題入力'!H165=1,'課題入力'!A165,"")</x:f>
       </x:c>
-      <x:c r="B165" s="113" t="str">
+      <x:c r="B165" s="142" t="str">
         <x:f>IF(A165="","",'課題入力'!B165)</x:f>
       </x:c>
-      <x:c r="C165" s="114" t="str">
+      <x:c r="C165" s="143" t="str">
         <x:f>IF(A165="","",'課題入力'!E165)</x:f>
       </x:c>
     </x:row>
-    <x:row r="166">
-      <x:c r="A166" s="112" t="str">
+    <x:row r="166" ht="24" customHeight="1">
+      <x:c r="A166" s="141" t="str">
         <x:f>IF('課題入力'!H166=1,'課題入力'!A166,"")</x:f>
       </x:c>
-      <x:c r="B166" s="113" t="str">
+      <x:c r="B166" s="142" t="str">
         <x:f>IF(A166="","",'課題入力'!B166)</x:f>
       </x:c>
-      <x:c r="C166" s="114" t="str">
+      <x:c r="C166" s="143" t="str">
         <x:f>IF(A166="","",'課題入力'!E166)</x:f>
       </x:c>
     </x:row>
-    <x:row r="167">
-      <x:c r="A167" s="112" t="str">
+    <x:row r="167" ht="24" customHeight="1">
+      <x:c r="A167" s="141" t="str">
         <x:f>IF('課題入力'!H167=1,'課題入力'!A167,"")</x:f>
       </x:c>
-      <x:c r="B167" s="113" t="str">
+      <x:c r="B167" s="142" t="str">
         <x:f>IF(A167="","",'課題入力'!B167)</x:f>
       </x:c>
-      <x:c r="C167" s="114" t="str">
+      <x:c r="C167" s="143" t="str">
         <x:f>IF(A167="","",'課題入力'!E167)</x:f>
       </x:c>
     </x:row>
-    <x:row r="168">
-      <x:c r="A168" s="112" t="str">
+    <x:row r="168" ht="24" customHeight="1">
+      <x:c r="A168" s="141" t="str">
         <x:f>IF('課題入力'!H168=1,'課題入力'!A168,"")</x:f>
       </x:c>
-      <x:c r="B168" s="113" t="str">
+      <x:c r="B168" s="142" t="str">
         <x:f>IF(A168="","",'課題入力'!B168)</x:f>
       </x:c>
-      <x:c r="C168" s="114" t="str">
+      <x:c r="C168" s="143" t="str">
         <x:f>IF(A168="","",'課題入力'!E168)</x:f>
       </x:c>
     </x:row>
-    <x:row r="169">
-      <x:c r="A169" s="112" t="str">
+    <x:row r="169" ht="24" customHeight="1">
+      <x:c r="A169" s="141" t="str">
         <x:f>IF('課題入力'!H169=1,'課題入力'!A169,"")</x:f>
       </x:c>
-      <x:c r="B169" s="113" t="str">
+      <x:c r="B169" s="142" t="str">
         <x:f>IF(A169="","",'課題入力'!B169)</x:f>
       </x:c>
-      <x:c r="C169" s="114" t="str">
+      <x:c r="C169" s="143" t="str">
         <x:f>IF(A169="","",'課題入力'!E169)</x:f>
       </x:c>
     </x:row>
-    <x:row r="170">
-      <x:c r="A170" s="112" t="str">
+    <x:row r="170" ht="24" customHeight="1">
+      <x:c r="A170" s="141" t="str">
         <x:f>IF('課題入力'!H170=1,'課題入力'!A170,"")</x:f>
       </x:c>
-      <x:c r="B170" s="113" t="str">
+      <x:c r="B170" s="142" t="str">
         <x:f>IF(A170="","",'課題入力'!B170)</x:f>
       </x:c>
-      <x:c r="C170" s="114" t="str">
+      <x:c r="C170" s="143" t="str">
         <x:f>IF(A170="","",'課題入力'!E170)</x:f>
       </x:c>
     </x:row>
-    <x:row r="171">
-      <x:c r="A171" s="112" t="str">
+    <x:row r="171" ht="24" customHeight="1">
+      <x:c r="A171" s="141" t="str">
         <x:f>IF('課題入力'!H171=1,'課題入力'!A171,"")</x:f>
       </x:c>
-      <x:c r="B171" s="113" t="str">
+      <x:c r="B171" s="142" t="str">
         <x:f>IF(A171="","",'課題入力'!B171)</x:f>
       </x:c>
-      <x:c r="C171" s="114" t="str">
+      <x:c r="C171" s="143" t="str">
         <x:f>IF(A171="","",'課題入力'!E171)</x:f>
       </x:c>
     </x:row>
-    <x:row r="172">
-      <x:c r="A172" s="112" t="str">
+    <x:row r="172" ht="24" customHeight="1">
+      <x:c r="A172" s="141" t="str">
         <x:f>IF('課題入力'!H172=1,'課題入力'!A172,"")</x:f>
       </x:c>
-      <x:c r="B172" s="113" t="str">
+      <x:c r="B172" s="142" t="str">
         <x:f>IF(A172="","",'課題入力'!B172)</x:f>
       </x:c>
-      <x:c r="C172" s="114" t="str">
+      <x:c r="C172" s="143" t="str">
         <x:f>IF(A172="","",'課題入力'!E172)</x:f>
       </x:c>
     </x:row>
-    <x:row r="173">
-      <x:c r="A173" s="112" t="str">
+    <x:row r="173" ht="24" customHeight="1">
+      <x:c r="A173" s="141" t="str">
         <x:f>IF('課題入力'!H173=1,'課題入力'!A173,"")</x:f>
       </x:c>
-      <x:c r="B173" s="113" t="str">
+      <x:c r="B173" s="142" t="str">
         <x:f>IF(A173="","",'課題入力'!B173)</x:f>
       </x:c>
-      <x:c r="C173" s="114" t="str">
+      <x:c r="C173" s="143" t="str">
         <x:f>IF(A173="","",'課題入力'!E173)</x:f>
       </x:c>
     </x:row>
-    <x:row r="174">
-      <x:c r="A174" s="112" t="str">
+    <x:row r="174" ht="24" customHeight="1">
+      <x:c r="A174" s="141" t="str">
         <x:f>IF('課題入力'!H174=1,'課題入力'!A174,"")</x:f>
       </x:c>
-      <x:c r="B174" s="113" t="str">
+      <x:c r="B174" s="142" t="str">
         <x:f>IF(A174="","",'課題入力'!B174)</x:f>
       </x:c>
-      <x:c r="C174" s="114" t="str">
+      <x:c r="C174" s="143" t="str">
         <x:f>IF(A174="","",'課題入力'!E174)</x:f>
       </x:c>
     </x:row>
-    <x:row r="175">
-      <x:c r="A175" s="112" t="str">
+    <x:row r="175" ht="24" customHeight="1">
+      <x:c r="A175" s="141" t="str">
         <x:f>IF('課題入力'!H175=1,'課題入力'!A175,"")</x:f>
       </x:c>
-      <x:c r="B175" s="113" t="str">
+      <x:c r="B175" s="142" t="str">
         <x:f>IF(A175="","",'課題入力'!B175)</x:f>
       </x:c>
-      <x:c r="C175" s="114" t="str">
+      <x:c r="C175" s="143" t="str">
         <x:f>IF(A175="","",'課題入力'!E175)</x:f>
       </x:c>
     </x:row>
-    <x:row r="176">
-      <x:c r="A176" s="112" t="str">
+    <x:row r="176" ht="24" customHeight="1">
+      <x:c r="A176" s="141" t="str">
         <x:f>IF('課題入力'!H176=1,'課題入力'!A176,"")</x:f>
       </x:c>
-      <x:c r="B176" s="113" t="str">
+      <x:c r="B176" s="142" t="str">
         <x:f>IF(A176="","",'課題入力'!B176)</x:f>
       </x:c>
-      <x:c r="C176" s="114" t="str">
+      <x:c r="C176" s="143" t="str">
         <x:f>IF(A176="","",'課題入力'!E176)</x:f>
       </x:c>
     </x:row>
-    <x:row r="177">
-      <x:c r="A177" s="112" t="str">
+    <x:row r="177" ht="24" customHeight="1">
+      <x:c r="A177" s="141" t="str">
         <x:f>IF('課題入力'!H177=1,'課題入力'!A177,"")</x:f>
       </x:c>
-      <x:c r="B177" s="113" t="str">
+      <x:c r="B177" s="142" t="str">
         <x:f>IF(A177="","",'課題入力'!B177)</x:f>
       </x:c>
-      <x:c r="C177" s="114" t="str">
+      <x:c r="C177" s="143" t="str">
         <x:f>IF(A177="","",'課題入力'!E177)</x:f>
       </x:c>
     </x:row>
-    <x:row r="178">
-      <x:c r="A178" s="112" t="str">
+    <x:row r="178" ht="24" customHeight="1">
+      <x:c r="A178" s="141" t="str">
         <x:f>IF('課題入力'!H178=1,'課題入力'!A178,"")</x:f>
       </x:c>
-      <x:c r="B178" s="113" t="str">
+      <x:c r="B178" s="142" t="str">
         <x:f>IF(A178="","",'課題入力'!B178)</x:f>
       </x:c>
-      <x:c r="C178" s="114" t="str">
+      <x:c r="C178" s="143" t="str">
         <x:f>IF(A178="","",'課題入力'!E178)</x:f>
       </x:c>
     </x:row>
-    <x:row r="179">
-      <x:c r="A179" s="112" t="str">
+    <x:row r="179" ht="24" customHeight="1">
+      <x:c r="A179" s="141" t="str">
         <x:f>IF('課題入力'!H179=1,'課題入力'!A179,"")</x:f>
       </x:c>
-      <x:c r="B179" s="113" t="str">
+      <x:c r="B179" s="142" t="str">
         <x:f>IF(A179="","",'課題入力'!B179)</x:f>
       </x:c>
-      <x:c r="C179" s="114" t="str">
+      <x:c r="C179" s="143" t="str">
         <x:f>IF(A179="","",'課題入力'!E179)</x:f>
       </x:c>
     </x:row>
-    <x:row r="180">
-      <x:c r="A180" s="112" t="str">
+    <x:row r="180" ht="24" customHeight="1">
+      <x:c r="A180" s="141" t="str">
         <x:f>IF('課題入力'!H180=1,'課題入力'!A180,"")</x:f>
       </x:c>
-      <x:c r="B180" s="113" t="str">
+      <x:c r="B180" s="142" t="str">
         <x:f>IF(A180="","",'課題入力'!B180)</x:f>
       </x:c>
-      <x:c r="C180" s="114" t="str">
+      <x:c r="C180" s="143" t="str">
         <x:f>IF(A180="","",'課題入力'!E180)</x:f>
       </x:c>
     </x:row>
-    <x:row r="181">
-      <x:c r="A181" s="112" t="str">
+    <x:row r="181" ht="24" customHeight="1">
+      <x:c r="A181" s="141" t="str">
         <x:f>IF('課題入力'!H181=1,'課題入力'!A181,"")</x:f>
       </x:c>
-      <x:c r="B181" s="113" t="str">
+      <x:c r="B181" s="142" t="str">
         <x:f>IF(A181="","",'課題入力'!B181)</x:f>
       </x:c>
-      <x:c r="C181" s="114" t="str">
+      <x:c r="C181" s="143" t="str">
         <x:f>IF(A181="","",'課題入力'!E181)</x:f>
       </x:c>
     </x:row>
-    <x:row r="182">
-      <x:c r="A182" s="112" t="str">
+    <x:row r="182" ht="24" customHeight="1">
+      <x:c r="A182" s="141" t="str">
         <x:f>IF('課題入力'!H182=1,'課題入力'!A182,"")</x:f>
       </x:c>
-      <x:c r="B182" s="113" t="str">
+      <x:c r="B182" s="142" t="str">
         <x:f>IF(A182="","",'課題入力'!B182)</x:f>
       </x:c>
-      <x:c r="C182" s="114" t="str">
+      <x:c r="C182" s="143" t="str">
         <x:f>IF(A182="","",'課題入力'!E182)</x:f>
       </x:c>
     </x:row>
-    <x:row r="183">
-      <x:c r="A183" s="112" t="str">
+    <x:row r="183" ht="24" customHeight="1">
+      <x:c r="A183" s="141" t="str">
         <x:f>IF('課題入力'!H183=1,'課題入力'!A183,"")</x:f>
       </x:c>
-      <x:c r="B183" s="113" t="str">
+      <x:c r="B183" s="142" t="str">
         <x:f>IF(A183="","",'課題入力'!B183)</x:f>
       </x:c>
-      <x:c r="C183" s="114" t="str">
+      <x:c r="C183" s="143" t="str">
         <x:f>IF(A183="","",'課題入力'!E183)</x:f>
       </x:c>
     </x:row>
-    <x:row r="184">
-      <x:c r="A184" s="112" t="str">
+    <x:row r="184" ht="24" customHeight="1">
+      <x:c r="A184" s="141" t="str">
         <x:f>IF('課題入力'!H184=1,'課題入力'!A184,"")</x:f>
       </x:c>
-      <x:c r="B184" s="113" t="str">
+      <x:c r="B184" s="142" t="str">
         <x:f>IF(A184="","",'課題入力'!B184)</x:f>
       </x:c>
-      <x:c r="C184" s="114" t="str">
+      <x:c r="C184" s="143" t="str">
         <x:f>IF(A184="","",'課題入力'!E184)</x:f>
       </x:c>
     </x:row>
-    <x:row r="185">
-      <x:c r="A185" s="112" t="str">
+    <x:row r="185" ht="24" customHeight="1">
+      <x:c r="A185" s="141" t="str">
         <x:f>IF('課題入力'!H185=1,'課題入力'!A185,"")</x:f>
       </x:c>
-      <x:c r="B185" s="113" t="str">
+      <x:c r="B185" s="142" t="str">
         <x:f>IF(A185="","",'課題入力'!B185)</x:f>
       </x:c>
-      <x:c r="C185" s="114" t="str">
+      <x:c r="C185" s="143" t="str">
         <x:f>IF(A185="","",'課題入力'!E185)</x:f>
       </x:c>
     </x:row>
-    <x:row r="186">
-      <x:c r="A186" s="112" t="str">
+    <x:row r="186" ht="24" customHeight="1">
+      <x:c r="A186" s="141" t="str">
         <x:f>IF('課題入力'!H186=1,'課題入力'!A186,"")</x:f>
       </x:c>
-      <x:c r="B186" s="113" t="str">
+      <x:c r="B186" s="142" t="str">
         <x:f>IF(A186="","",'課題入力'!B186)</x:f>
       </x:c>
-      <x:c r="C186" s="114" t="str">
+      <x:c r="C186" s="143" t="str">
         <x:f>IF(A186="","",'課題入力'!E186)</x:f>
       </x:c>
     </x:row>
-    <x:row r="187">
-      <x:c r="A187" s="112" t="str">
+    <x:row r="187" ht="24" customHeight="1">
+      <x:c r="A187" s="141" t="str">
         <x:f>IF('課題入力'!H187=1,'課題入力'!A187,"")</x:f>
       </x:c>
-      <x:c r="B187" s="113" t="str">
+      <x:c r="B187" s="142" t="str">
         <x:f>IF(A187="","",'課題入力'!B187)</x:f>
       </x:c>
-      <x:c r="C187" s="114" t="str">
+      <x:c r="C187" s="143" t="str">
         <x:f>IF(A187="","",'課題入力'!E187)</x:f>
       </x:c>
     </x:row>
-    <x:row r="188">
-      <x:c r="A188" s="112" t="str">
+    <x:row r="188" ht="24" customHeight="1">
+      <x:c r="A188" s="141" t="str">
         <x:f>IF('課題入力'!H188=1,'課題入力'!A188,"")</x:f>
       </x:c>
-      <x:c r="B188" s="113" t="str">
+      <x:c r="B188" s="142" t="str">
         <x:f>IF(A188="","",'課題入力'!B188)</x:f>
       </x:c>
-      <x:c r="C188" s="114" t="str">
+      <x:c r="C188" s="143" t="str">
         <x:f>IF(A188="","",'課題入力'!E188)</x:f>
       </x:c>
     </x:row>
-    <x:row r="189">
-      <x:c r="A189" s="112" t="str">
+    <x:row r="189" ht="24" customHeight="1">
+      <x:c r="A189" s="141" t="str">
         <x:f>IF('課題入力'!H189=1,'課題入力'!A189,"")</x:f>
       </x:c>
-      <x:c r="B189" s="113" t="str">
+      <x:c r="B189" s="142" t="str">
         <x:f>IF(A189="","",'課題入力'!B189)</x:f>
       </x:c>
-      <x:c r="C189" s="114" t="str">
+      <x:c r="C189" s="143" t="str">
         <x:f>IF(A189="","",'課題入力'!E189)</x:f>
       </x:c>
     </x:row>
-    <x:row r="190">
-      <x:c r="A190" s="112" t="str">
+    <x:row r="190" ht="24" customHeight="1">
+      <x:c r="A190" s="141" t="str">
         <x:f>IF('課題入力'!H190=1,'課題入力'!A190,"")</x:f>
       </x:c>
-      <x:c r="B190" s="113" t="str">
+      <x:c r="B190" s="142" t="str">
         <x:f>IF(A190="","",'課題入力'!B190)</x:f>
       </x:c>
-      <x:c r="C190" s="114" t="str">
+      <x:c r="C190" s="143" t="str">
         <x:f>IF(A190="","",'課題入力'!E190)</x:f>
       </x:c>
     </x:row>
-    <x:row r="191">
-      <x:c r="A191" s="112" t="str">
+    <x:row r="191" ht="24" customHeight="1">
+      <x:c r="A191" s="141" t="str">
         <x:f>IF('課題入力'!H191=1,'課題入力'!A191,"")</x:f>
       </x:c>
-      <x:c r="B191" s="113" t="str">
+      <x:c r="B191" s="142" t="str">
         <x:f>IF(A191="","",'課題入力'!B191)</x:f>
       </x:c>
-      <x:c r="C191" s="114" t="str">
+      <x:c r="C191" s="143" t="str">
         <x:f>IF(A191="","",'課題入力'!E191)</x:f>
       </x:c>
     </x:row>
-    <x:row r="192">
-      <x:c r="A192" s="112" t="str">
+    <x:row r="192" ht="24" customHeight="1">
+      <x:c r="A192" s="141" t="str">
         <x:f>IF('課題入力'!H192=1,'課題入力'!A192,"")</x:f>
       </x:c>
-      <x:c r="B192" s="113" t="str">
+      <x:c r="B192" s="142" t="str">
         <x:f>IF(A192="","",'課題入力'!B192)</x:f>
       </x:c>
-      <x:c r="C192" s="114" t="str">
+      <x:c r="C192" s="143" t="str">
         <x:f>IF(A192="","",'課題入力'!E192)</x:f>
       </x:c>
     </x:row>
-    <x:row r="193">
-      <x:c r="A193" s="112" t="str">
+    <x:row r="193" ht="24" customHeight="1">
+      <x:c r="A193" s="141" t="str">
         <x:f>IF('課題入力'!H193=1,'課題入力'!A193,"")</x:f>
       </x:c>
-      <x:c r="B193" s="113" t="str">
+      <x:c r="B193" s="142" t="str">
         <x:f>IF(A193="","",'課題入力'!B193)</x:f>
       </x:c>
-      <x:c r="C193" s="114" t="str">
+      <x:c r="C193" s="143" t="str">
         <x:f>IF(A193="","",'課題入力'!E193)</x:f>
       </x:c>
     </x:row>
-    <x:row r="194">
-      <x:c r="A194" s="112" t="str">
+    <x:row r="194" ht="24" customHeight="1">
+      <x:c r="A194" s="141" t="str">
         <x:f>IF('課題入力'!H194=1,'課題入力'!A194,"")</x:f>
       </x:c>
-      <x:c r="B194" s="113" t="str">
+      <x:c r="B194" s="142" t="str">
         <x:f>IF(A194="","",'課題入力'!B194)</x:f>
       </x:c>
-      <x:c r="C194" s="114" t="str">
+      <x:c r="C194" s="143" t="str">
         <x:f>IF(A194="","",'課題入力'!E194)</x:f>
       </x:c>
     </x:row>
-    <x:row r="195">
-      <x:c r="A195" s="112" t="str">
+    <x:row r="195" ht="24" customHeight="1">
+      <x:c r="A195" s="141" t="str">
         <x:f>IF('課題入力'!H195=1,'課題入力'!A195,"")</x:f>
       </x:c>
-      <x:c r="B195" s="113" t="str">
+      <x:c r="B195" s="142" t="str">
         <x:f>IF(A195="","",'課題入力'!B195)</x:f>
       </x:c>
-      <x:c r="C195" s="114" t="str">
+      <x:c r="C195" s="143" t="str">
         <x:f>IF(A195="","",'課題入力'!E195)</x:f>
       </x:c>
     </x:row>
-    <x:row r="196">
-      <x:c r="A196" s="112" t="str">
+    <x:row r="196" ht="24" customHeight="1">
+      <x:c r="A196" s="141" t="str">
         <x:f>IF('課題入力'!H196=1,'課題入力'!A196,"")</x:f>
       </x:c>
-      <x:c r="B196" s="113" t="str">
+      <x:c r="B196" s="142" t="str">
         <x:f>IF(A196="","",'課題入力'!B196)</x:f>
       </x:c>
-      <x:c r="C196" s="114" t="str">
+      <x:c r="C196" s="143" t="str">
         <x:f>IF(A196="","",'課題入力'!E196)</x:f>
       </x:c>
     </x:row>
-    <x:row r="197">
-      <x:c r="A197" s="112" t="str">
+    <x:row r="197" ht="24" customHeight="1">
+      <x:c r="A197" s="141" t="str">
         <x:f>IF('課題入力'!H197=1,'課題入力'!A197,"")</x:f>
       </x:c>
-      <x:c r="B197" s="113" t="str">
+      <x:c r="B197" s="142" t="str">
         <x:f>IF(A197="","",'課題入力'!B197)</x:f>
       </x:c>
-      <x:c r="C197" s="114" t="str">
+      <x:c r="C197" s="143" t="str">
         <x:f>IF(A197="","",'課題入力'!E197)</x:f>
       </x:c>
     </x:row>
-    <x:row r="198">
-      <x:c r="A198" s="112" t="str">
+    <x:row r="198" ht="24" customHeight="1">
+      <x:c r="A198" s="141" t="str">
         <x:f>IF('課題入力'!H198=1,'課題入力'!A198,"")</x:f>
       </x:c>
-      <x:c r="B198" s="113" t="str">
+      <x:c r="B198" s="142" t="str">
         <x:f>IF(A198="","",'課題入力'!B198)</x:f>
       </x:c>
-      <x:c r="C198" s="114" t="str">
+      <x:c r="C198" s="143" t="str">
         <x:f>IF(A198="","",'課題入力'!E198)</x:f>
       </x:c>
     </x:row>
-    <x:row r="199">
-      <x:c r="A199" s="112" t="str">
+    <x:row r="199" ht="24" customHeight="1">
+      <x:c r="A199" s="141" t="str">
         <x:f>IF('課題入力'!H199=1,'課題入力'!A199,"")</x:f>
       </x:c>
-      <x:c r="B199" s="113" t="str">
+      <x:c r="B199" s="142" t="str">
         <x:f>IF(A199="","",'課題入力'!B199)</x:f>
       </x:c>
-      <x:c r="C199" s="114" t="str">
+      <x:c r="C199" s="143" t="str">
         <x:f>IF(A199="","",'課題入力'!E199)</x:f>
       </x:c>
     </x:row>
-    <x:row r="200">
-      <x:c r="A200" s="112" t="str">
+    <x:row r="200" ht="24" customHeight="1">
+      <x:c r="A200" s="141" t="str">
         <x:f>IF('課題入力'!H200=1,'課題入力'!A200,"")</x:f>
       </x:c>
-      <x:c r="B200" s="113" t="str">
+      <x:c r="B200" s="142" t="str">
         <x:f>IF(A200="","",'課題入力'!B200)</x:f>
       </x:c>
-      <x:c r="C200" s="114" t="str">
+      <x:c r="C200" s="143" t="str">
         <x:f>IF(A200="","",'課題入力'!E200)</x:f>
       </x:c>
     </x:row>
-    <x:row r="201">
-      <x:c r="A201" s="112" t="str">
+    <x:row r="201" ht="24" customHeight="1">
+      <x:c r="A201" s="141" t="str">
         <x:f>IF('課題入力'!H201=1,'課題入力'!A201,"")</x:f>
       </x:c>
-      <x:c r="B201" s="113" t="str">
+      <x:c r="B201" s="142" t="str">
         <x:f>IF(A201="","",'課題入力'!B201)</x:f>
       </x:c>
-      <x:c r="C201" s="114" t="str">
+      <x:c r="C201" s="143" t="str">
         <x:f>IF(A201="","",'課題入力'!E201)</x:f>
       </x:c>
     </x:row>
-    <x:row r="202">
-      <x:c r="A202" s="112" t="str">
+    <x:row r="202" ht="24" customHeight="1">
+      <x:c r="A202" s="141" t="str">
         <x:f>IF('課題入力'!H202=1,'課題入力'!A202,"")</x:f>
       </x:c>
-      <x:c r="B202" s="113" t="str">
+      <x:c r="B202" s="142" t="str">
         <x:f>IF(A202="","",'課題入力'!B202)</x:f>
       </x:c>
-      <x:c r="C202" s="114" t="str">
+      <x:c r="C202" s="143" t="str">
         <x:f>IF(A202="","",'課題入力'!E202)</x:f>
       </x:c>
     </x:row>
-    <x:row r="203">
-      <x:c r="A203" s="112" t="str">
+    <x:row r="203" ht="24" customHeight="1">
+      <x:c r="A203" s="141" t="str">
         <x:f>IF('課題入力'!H203=1,'課題入力'!A203,"")</x:f>
       </x:c>
-      <x:c r="B203" s="113" t="str">
+      <x:c r="B203" s="142" t="str">
         <x:f>IF(A203="","",'課題入力'!B203)</x:f>
       </x:c>
-      <x:c r="C203" s="114" t="str">
+      <x:c r="C203" s="143" t="str">
         <x:f>IF(A203="","",'課題入力'!E203)</x:f>
       </x:c>
     </x:row>
-    <x:row r="204">
-      <x:c r="A204" s="112" t="str">
+    <x:row r="204" ht="24" customHeight="1">
+      <x:c r="A204" s="141" t="str">
         <x:f>IF('課題入力'!H204=1,'課題入力'!A204,"")</x:f>
       </x:c>
-      <x:c r="B204" s="113" t="str">
+      <x:c r="B204" s="142" t="str">
         <x:f>IF(A204="","",'課題入力'!B204)</x:f>
       </x:c>
-      <x:c r="C204" s="114" t="str">
+      <x:c r="C204" s="143" t="str">
         <x:f>IF(A204="","",'課題入力'!E204)</x:f>
       </x:c>
     </x:row>
-    <x:row r="205">
-      <x:c r="A205" s="112" t="str">
+    <x:row r="205" ht="24" customHeight="1">
+      <x:c r="A205" s="141" t="str">
         <x:f>IF('課題入力'!H205=1,'課題入力'!A205,"")</x:f>
       </x:c>
-      <x:c r="B205" s="113" t="str">
+      <x:c r="B205" s="142" t="str">
         <x:f>IF(A205="","",'課題入力'!B205)</x:f>
       </x:c>
-      <x:c r="C205" s="114" t="str">
+      <x:c r="C205" s="143" t="str">
         <x:f>IF(A205="","",'課題入力'!E205)</x:f>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A3:C3"/>
+    <x:mergeCell ref="A2:C2"/>
+    <x:mergeCell ref="A3:C4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>